<commit_message>
Balance Wayground answer distribution
</commit_message>
<xml_diff>
--- a/xlsx/SEL平板暖身題庫_Wayground.xlsx
+++ b/xlsx/SEL平板暖身題庫_Wayground.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wayground匯入題庫" sheetId="1" r:id="R237f6ff4c7ac4011"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="教師備課對照" sheetId="2" r:id="R8aeb2b0de1574723"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用說明" sheetId="3" r:id="Rfd98f5914649446c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wayground匯入題庫" sheetId="1" r:id="Raff7737c0c1c44e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="教師備課對照" sheetId="2" r:id="R63e7fc4cbc554e6c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用說明" sheetId="3" r:id="R33820b08457d4353"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -416,10 +416,10 @@
         <x:v>Multiple Choice</x:v>
       </x:c>
       <x:c r="C2" s="11" t="str">
+        <x:v>陰天</x:v>
+      </x:c>
+      <x:c r="D2" s="11" t="str">
         <x:v>晴天</x:v>
-      </x:c>
-      <x:c r="D2" s="11" t="str">
-        <x:v>陰天</x:v>
       </x:c>
       <x:c r="E2" s="11" t="str">
         <x:v>下雨</x:v>
@@ -429,7 +429,7 @@
       </x:c>
       <x:c r="G2" s="11" t="str"/>
       <x:c r="H2" s="11" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="I2" s="11" t="n">
         <x:v>30</x:v>
@@ -478,20 +478,20 @@
         <x:v>Multiple Choice</x:v>
       </x:c>
       <x:c r="C4" s="11" t="str">
+        <x:v>大聲詢問細節</x:v>
+      </x:c>
+      <x:c r="D4" s="11" t="str">
+        <x:v>取笑對方</x:v>
+      </x:c>
+      <x:c r="E4" s="11" t="str">
         <x:v>安靜陪伴並通知可信任的大人</x:v>
-      </x:c>
-      <x:c r="D4" s="11" t="str">
-        <x:v>大聲詢問細節</x:v>
-      </x:c>
-      <x:c r="E4" s="11" t="str">
-        <x:v>取笑對方</x:v>
       </x:c>
       <x:c r="F4" s="11" t="str">
         <x:v>拍照傳到群組</x:v>
       </x:c>
       <x:c r="G4" s="11" t="str"/>
       <x:c r="H4" s="11" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="I4" s="11" t="n">
         <x:v>30</x:v>
@@ -509,20 +509,20 @@
         <x:v>Multiple Choice</x:v>
       </x:c>
       <x:c r="C5" s="11" t="str">
+        <x:v>沒有固定答案，察覺自己需要時就可以停</x:v>
+      </x:c>
+      <x:c r="D5" s="11" t="str">
         <x:v>1 度</x:v>
       </x:c>
-      <x:c r="D5" s="11" t="str">
+      <x:c r="E5" s="11" t="str">
         <x:v>2 度</x:v>
       </x:c>
-      <x:c r="E5" s="11" t="str">
+      <x:c r="F5" s="11" t="str">
         <x:v>3 度以上</x:v>
-      </x:c>
-      <x:c r="F5" s="11" t="str">
-        <x:v>沒有固定答案，察覺自己需要時就可以停</x:v>
       </x:c>
       <x:c r="G5" s="11" t="str"/>
       <x:c r="H5" s="11" t="n">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I5" s="11" t="n">
         <x:v>30</x:v>
@@ -540,20 +540,20 @@
         <x:v>Multiple Choice</x:v>
       </x:c>
       <x:c r="C6" s="11" t="str">
+        <x:v>完全不告訴任何人</x:v>
+      </x:c>
+      <x:c r="D6" s="11" t="str">
+        <x:v>只在網路上找陌生人</x:v>
+      </x:c>
+      <x:c r="E6" s="11" t="str">
+        <x:v>責怪自己不夠勇敢</x:v>
+      </x:c>
+      <x:c r="F6" s="11" t="str">
         <x:v>可信任的導師、家人、校護或輔導老師</x:v>
-      </x:c>
-      <x:c r="D6" s="11" t="str">
-        <x:v>完全不告訴任何人</x:v>
-      </x:c>
-      <x:c r="E6" s="11" t="str">
-        <x:v>只在網路上找陌生人</x:v>
-      </x:c>
-      <x:c r="F6" s="11" t="str">
-        <x:v>責怪自己不夠勇敢</x:v>
       </x:c>
       <x:c r="G6" s="11" t="str"/>
       <x:c r="H6" s="11" t="n">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="I6" s="11" t="n">
         <x:v>30</x:v>
@@ -571,10 +571,10 @@
         <x:v>Multiple Choice</x:v>
       </x:c>
       <x:c r="C7" s="11" t="str">
+        <x:v>逼對方改變</x:v>
+      </x:c>
+      <x:c r="D7" s="11" t="str">
         <x:v>說出自己的喜好，也聽聽對方的想法</x:v>
-      </x:c>
-      <x:c r="D7" s="11" t="str">
-        <x:v>逼對方改變</x:v>
       </x:c>
       <x:c r="E7" s="11" t="str">
         <x:v>嘲笑對方</x:v>
@@ -584,7 +584,7 @@
       </x:c>
       <x:c r="G7" s="11" t="str"/>
       <x:c r="H7" s="11" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="I7" s="11" t="n">
         <x:v>30</x:v>
@@ -602,20 +602,20 @@
         <x:v>Multiple Choice</x:v>
       </x:c>
       <x:c r="C8" s="11" t="str">
+        <x:v>好啦，大家都傳了</x:v>
+      </x:c>
+      <x:c r="D8" s="11" t="str">
+        <x:v>你不傳我就取笑你</x:v>
+      </x:c>
+      <x:c r="E8" s="11" t="str">
         <x:v>我不想分享這張照片，請不要傳</x:v>
-      </x:c>
-      <x:c r="D8" s="11" t="str">
-        <x:v>好啦，大家都傳了</x:v>
-      </x:c>
-      <x:c r="E8" s="11" t="str">
-        <x:v>你不傳我就取笑你</x:v>
       </x:c>
       <x:c r="F8" s="11" t="str">
         <x:v>先傳給陌生人問問看</x:v>
       </x:c>
       <x:c r="G8" s="11" t="str"/>
       <x:c r="H8" s="11" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="I8" s="11" t="n">
         <x:v>30</x:v>
@@ -664,10 +664,10 @@
         <x:v>Multiple Choice</x:v>
       </x:c>
       <x:c r="C10" s="11" t="str">
+        <x:v>你一定要現在回答</x:v>
+      </x:c>
+      <x:c r="D10" s="11" t="str">
         <x:v>你想先聽聽他的想法嗎？也可以等一下再說</x:v>
-      </x:c>
-      <x:c r="D10" s="11" t="str">
-        <x:v>你一定要現在回答</x:v>
       </x:c>
       <x:c r="E10" s="11" t="str">
         <x:v>大家不要理他</x:v>
@@ -677,7 +677,7 @@
       </x:c>
       <x:c r="G10" s="11" t="str"/>
       <x:c r="H10" s="11" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="I10" s="11" t="n">
         <x:v>30</x:v>
@@ -695,20 +695,20 @@
         <x:v>Multiple Choice</x:v>
       </x:c>
       <x:c r="C11" s="11" t="str">
+        <x:v>只要朋友開心就好</x:v>
+      </x:c>
+      <x:c r="D11" s="11" t="str">
+        <x:v>別人怎麼做我就怎麼做</x:v>
+      </x:c>
+      <x:c r="E11" s="11" t="str">
+        <x:v>答應後再說</x:v>
+      </x:c>
+      <x:c r="F11" s="11" t="str">
         <x:v>我的感受、我的界線和可能的結果</x:v>
-      </x:c>
-      <x:c r="D11" s="11" t="str">
-        <x:v>只要朋友開心就好</x:v>
-      </x:c>
-      <x:c r="E11" s="11" t="str">
-        <x:v>別人怎麼做我就怎麼做</x:v>
-      </x:c>
-      <x:c r="F11" s="11" t="str">
-        <x:v>答應後再說</x:v>
       </x:c>
       <x:c r="G11" s="11" t="str"/>
       <x:c r="H11" s="11" t="n">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="I11" s="11" t="n">
         <x:v>30</x:v>
@@ -732,14 +732,14 @@
         <x:v>日期</x:v>
       </x:c>
       <x:c r="E12" s="11" t="str">
+        <x:v>以上都要查</x:v>
+      </x:c>
+      <x:c r="F12" s="11" t="str">
         <x:v>證據</x:v>
-      </x:c>
-      <x:c r="F12" s="11" t="str">
-        <x:v>以上都要查</x:v>
       </x:c>
       <x:c r="G12" s="11" t="str"/>
       <x:c r="H12" s="11" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="I12" s="11" t="n">
         <x:v>30</x:v>
@@ -788,20 +788,20 @@
         <x:v>Multiple Choice</x:v>
       </x:c>
       <x:c r="C14" s="11" t="str">
+        <x:v>夠快嗎？夠酸嗎？會紅嗎？</x:v>
+      </x:c>
+      <x:c r="D14" s="11" t="str">
+        <x:v>大家按讚嗎？有趣嗎？刺激嗎？</x:v>
+      </x:c>
+      <x:c r="E14" s="11" t="str">
+        <x:v>可以匿名嗎？可以刪掉嗎？可以轉傳嗎？</x:v>
+      </x:c>
+      <x:c r="F14" s="11" t="str">
         <x:v>是真的嗎？必要嗎？尊重嗎？</x:v>
-      </x:c>
-      <x:c r="D14" s="11" t="str">
-        <x:v>夠快嗎？夠酸嗎？會紅嗎？</x:v>
-      </x:c>
-      <x:c r="E14" s="11" t="str">
-        <x:v>大家按讚嗎？有趣嗎？刺激嗎？</x:v>
-      </x:c>
-      <x:c r="F14" s="11" t="str">
-        <x:v>可以匿名嗎？可以刪掉嗎？可以轉傳嗎？</x:v>
       </x:c>
       <x:c r="G14" s="11" t="str"/>
       <x:c r="H14" s="11" t="n">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="I14" s="11" t="n">
         <x:v>30</x:v>
@@ -822,17 +822,17 @@
         <x:v>眼睛疲累</x:v>
       </x:c>
       <x:c r="D15" s="11" t="str">
+        <x:v>以上都可能</x:v>
+      </x:c>
+      <x:c r="E15" s="11" t="str">
         <x:v>睡不著</x:v>
       </x:c>
-      <x:c r="E15" s="11" t="str">
+      <x:c r="F15" s="11" t="str">
         <x:v>心情變差</x:v>
-      </x:c>
-      <x:c r="F15" s="11" t="str">
-        <x:v>以上都可能</x:v>
       </x:c>
       <x:c r="G15" s="11" t="str"/>
       <x:c r="H15" s="11" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="I15" s="11" t="n">
         <x:v>30</x:v>
@@ -887,14 +887,14 @@
         <x:v>睡不好</x:v>
       </x:c>
       <x:c r="E17" s="11" t="str">
+        <x:v>以上都可能</x:v>
+      </x:c>
+      <x:c r="F17" s="11" t="str">
         <x:v>一直擔心來不及</x:v>
-      </x:c>
-      <x:c r="F17" s="11" t="str">
-        <x:v>以上都可能</x:v>
       </x:c>
       <x:c r="G17" s="11" t="str"/>
       <x:c r="H17" s="11" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="I17" s="11" t="n">
         <x:v>30</x:v>
@@ -912,20 +912,20 @@
         <x:v>Multiple Choice</x:v>
       </x:c>
       <x:c r="C18" s="11" t="str">
+        <x:v>永遠第一名</x:v>
+      </x:c>
+      <x:c r="D18" s="11" t="str">
+        <x:v>不要失敗</x:v>
+      </x:c>
+      <x:c r="E18" s="11" t="str">
+        <x:v>讓所有人都滿意</x:v>
+      </x:c>
+      <x:c r="F18" s="11" t="str">
         <x:v>今天完成 15 分鐘複習</x:v>
-      </x:c>
-      <x:c r="D18" s="11" t="str">
-        <x:v>永遠第一名</x:v>
-      </x:c>
-      <x:c r="E18" s="11" t="str">
-        <x:v>不要失敗</x:v>
-      </x:c>
-      <x:c r="F18" s="11" t="str">
-        <x:v>讓所有人都滿意</x:v>
       </x:c>
       <x:c r="G18" s="11" t="str"/>
       <x:c r="H18" s="11" t="n">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="I18" s="11" t="n">
         <x:v>30</x:v>
@@ -974,10 +974,10 @@
         <x:v>Multiple Choice</x:v>
       </x:c>
       <x:c r="C20" s="11" t="str">
+        <x:v>只要求你忍耐的人</x:v>
+      </x:c>
+      <x:c r="D20" s="11" t="str">
         <x:v>願意聽、尊重界線並一起找方法的人</x:v>
-      </x:c>
-      <x:c r="D20" s="11" t="str">
-        <x:v>只要求你忍耐的人</x:v>
       </x:c>
       <x:c r="E20" s="11" t="str">
         <x:v>會把秘密公開的人</x:v>
@@ -987,7 +987,7 @@
       </x:c>
       <x:c r="G20" s="11" t="str"/>
       <x:c r="H20" s="11" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="I20" s="11" t="n">
         <x:v>30</x:v>
@@ -1011,14 +1011,14 @@
         <x:v>遇到困擾時找可信任的大人</x:v>
       </x:c>
       <x:c r="E21" s="11" t="str">
+        <x:v>以上都可以，選一個明天先試</x:v>
+      </x:c>
+      <x:c r="F21" s="11" t="str">
         <x:v>先查證再轉傳訊息</x:v>
-      </x:c>
-      <x:c r="F21" s="11" t="str">
-        <x:v>以上都可以，選一個明天先試</x:v>
       </x:c>
       <x:c r="G21" s="11" t="str"/>
       <x:c r="H21" s="11" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="I21" s="11" t="n">
         <x:v>30</x:v>
@@ -1031,7 +1031,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7455ba80d2ab45fe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra9d7b4976bac497c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1095,10 +1095,10 @@
         <x:v>辨識當下情緒，不要求分享個人秘密。</x:v>
       </x:c>
       <x:c r="D2" s="11" t="str">
+        <x:v>陰天</x:v>
+      </x:c>
+      <x:c r="E2" s="11" t="str">
         <x:v>晴天</x:v>
-      </x:c>
-      <x:c r="E2" s="11" t="str">
-        <x:v>陰天</x:v>
       </x:c>
       <x:c r="F2" s="11" t="str">
         <x:v>下雨</x:v>
@@ -1107,7 +1107,7 @@
         <x:v>雷雨</x:v>
       </x:c>
       <x:c r="H2" s="11" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="I2" s="11" t="n">
         <x:v>30</x:v>
@@ -1139,7 +1139,7 @@
         <x:v>以上都可能</x:v>
       </x:c>
       <x:c r="H3" s="11" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="I3" s="11" t="n">
         <x:v>30</x:v>
@@ -1159,13 +1159,13 @@
         <x:v>練習青春期與生理期的尊重和求助。</x:v>
       </x:c>
       <x:c r="D4" s="11" t="str">
+        <x:v>大聲詢問細節</x:v>
+      </x:c>
+      <x:c r="E4" s="11" t="str">
+        <x:v>取笑對方</x:v>
+      </x:c>
+      <x:c r="F4" s="11" t="str">
         <x:v>安靜陪伴並通知可信任的大人</x:v>
-      </x:c>
-      <x:c r="E4" s="11" t="str">
-        <x:v>大聲詢問細節</x:v>
-      </x:c>
-      <x:c r="F4" s="11" t="str">
-        <x:v>取笑對方</x:v>
       </x:c>
       <x:c r="G4" s="11" t="str">
         <x:v>拍照傳到群組</x:v>
@@ -1191,19 +1191,19 @@
         <x:v>察覺需要暫停的時機。</x:v>
       </x:c>
       <x:c r="D5" s="11" t="str">
+        <x:v>沒有固定答案，察覺自己需要時就可以停</x:v>
+      </x:c>
+      <x:c r="E5" s="11" t="str">
         <x:v>1 度</x:v>
       </x:c>
-      <x:c r="E5" s="11" t="str">
+      <x:c r="F5" s="11" t="str">
         <x:v>2 度</x:v>
       </x:c>
-      <x:c r="F5" s="11" t="str">
+      <x:c r="G5" s="11" t="str">
         <x:v>3 度以上</x:v>
       </x:c>
-      <x:c r="G5" s="11" t="str">
-        <x:v>沒有固定答案，察覺自己需要時就可以停</x:v>
-      </x:c>
       <x:c r="H5" s="11" t="n">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I5" s="11" t="n">
         <x:v>30</x:v>
@@ -1223,19 +1223,19 @@
         <x:v>建立可信任的求助入口。</x:v>
       </x:c>
       <x:c r="D6" s="11" t="str">
+        <x:v>完全不告訴任何人</x:v>
+      </x:c>
+      <x:c r="E6" s="11" t="str">
+        <x:v>只在網路上找陌生人</x:v>
+      </x:c>
+      <x:c r="F6" s="11" t="str">
+        <x:v>責怪自己不夠勇敢</x:v>
+      </x:c>
+      <x:c r="G6" s="11" t="str">
         <x:v>可信任的導師、家人、校護或輔導老師</x:v>
       </x:c>
-      <x:c r="E6" s="11" t="str">
-        <x:v>完全不告訴任何人</x:v>
-      </x:c>
-      <x:c r="F6" s="11" t="str">
-        <x:v>只在網路上找陌生人</x:v>
-      </x:c>
-      <x:c r="G6" s="11" t="str">
-        <x:v>責怪自己不夠勇敢</x:v>
-      </x:c>
       <x:c r="H6" s="11" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="I6" s="11" t="n">
         <x:v>30</x:v>
@@ -1255,10 +1255,10 @@
         <x:v>尊重友誼中的差異。</x:v>
       </x:c>
       <x:c r="D7" s="11" t="str">
+        <x:v>逼對方改變</x:v>
+      </x:c>
+      <x:c r="E7" s="11" t="str">
         <x:v>說出自己的喜好，也聽聽對方的想法</x:v>
-      </x:c>
-      <x:c r="E7" s="11" t="str">
-        <x:v>逼對方改變</x:v>
       </x:c>
       <x:c r="F7" s="11" t="str">
         <x:v>嘲笑對方</x:v>
@@ -1267,7 +1267,7 @@
         <x:v>假裝自己什麼都喜歡</x:v>
       </x:c>
       <x:c r="H7" s="11" t="n">
-        <x:v>6</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="I7" s="11" t="n">
         <x:v>30</x:v>
@@ -1287,19 +1287,19 @@
         <x:v>練習影像與個人界線。</x:v>
       </x:c>
       <x:c r="D8" s="11" t="str">
+        <x:v>好啦，大家都傳了</x:v>
+      </x:c>
+      <x:c r="E8" s="11" t="str">
+        <x:v>你不傳我就取笑你</x:v>
+      </x:c>
+      <x:c r="F8" s="11" t="str">
         <x:v>我不想分享這張照片，請不要傳</x:v>
-      </x:c>
-      <x:c r="E8" s="11" t="str">
-        <x:v>好啦，大家都傳了</x:v>
-      </x:c>
-      <x:c r="F8" s="11" t="str">
-        <x:v>你不傳我就取笑你</x:v>
       </x:c>
       <x:c r="G8" s="11" t="str">
         <x:v>先傳給陌生人問問看</x:v>
       </x:c>
       <x:c r="H8" s="11" t="n">
-        <x:v>7</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="I8" s="11" t="n">
         <x:v>30</x:v>
@@ -1331,7 +1331,7 @@
         <x:v>立刻把爭吵內容轉傳</x:v>
       </x:c>
       <x:c r="H9" s="11" t="n">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I9" s="11" t="n">
         <x:v>30</x:v>
@@ -1351,10 +1351,10 @@
         <x:v>練習不強迫的團體邀請。</x:v>
       </x:c>
       <x:c r="D10" s="11" t="str">
+        <x:v>你一定要現在回答</x:v>
+      </x:c>
+      <x:c r="E10" s="11" t="str">
         <x:v>你想先聽聽他的想法嗎？也可以等一下再說</x:v>
-      </x:c>
-      <x:c r="E10" s="11" t="str">
-        <x:v>你一定要現在回答</x:v>
       </x:c>
       <x:c r="F10" s="11" t="str">
         <x:v>大家不要理他</x:v>
@@ -1363,7 +1363,7 @@
         <x:v>替他直接決定</x:v>
       </x:c>
       <x:c r="H10" s="11" t="n">
-        <x:v>9</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="I10" s="11" t="n">
         <x:v>30</x:v>
@@ -1383,19 +1383,19 @@
         <x:v>整合表達、拒絕與決定的方法。</x:v>
       </x:c>
       <x:c r="D11" s="11" t="str">
+        <x:v>只要朋友開心就好</x:v>
+      </x:c>
+      <x:c r="E11" s="11" t="str">
+        <x:v>別人怎麼做我就怎麼做</x:v>
+      </x:c>
+      <x:c r="F11" s="11" t="str">
+        <x:v>答應後再說</x:v>
+      </x:c>
+      <x:c r="G11" s="11" t="str">
         <x:v>我的感受、我的界線和可能的結果</x:v>
       </x:c>
-      <x:c r="E11" s="11" t="str">
-        <x:v>只要朋友開心就好</x:v>
-      </x:c>
-      <x:c r="F11" s="11" t="str">
-        <x:v>別人怎麼做我就怎麼做</x:v>
-      </x:c>
-      <x:c r="G11" s="11" t="str">
-        <x:v>答應後再說</x:v>
-      </x:c>
       <x:c r="H11" s="11" t="n">
-        <x:v>10</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="I11" s="11" t="n">
         <x:v>30</x:v>
@@ -1421,13 +1421,13 @@
         <x:v>日期</x:v>
       </x:c>
       <x:c r="F12" s="11" t="str">
+        <x:v>以上都要查</x:v>
+      </x:c>
+      <x:c r="G12" s="11" t="str">
         <x:v>證據</x:v>
       </x:c>
-      <x:c r="G12" s="11" t="str">
-        <x:v>以上都要查</x:v>
-      </x:c>
       <x:c r="H12" s="11" t="n">
-        <x:v>11</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="I12" s="11" t="n">
         <x:v>30</x:v>
@@ -1459,7 +1459,7 @@
         <x:v>喜歡的食物</x:v>
       </x:c>
       <x:c r="H13" s="11" t="n">
-        <x:v>12</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I13" s="11" t="n">
         <x:v>30</x:v>
@@ -1479,19 +1479,19 @@
         <x:v>練習數位同理與負責任留言。</x:v>
       </x:c>
       <x:c r="D14" s="11" t="str">
+        <x:v>夠快嗎？夠酸嗎？會紅嗎？</x:v>
+      </x:c>
+      <x:c r="E14" s="11" t="str">
+        <x:v>大家按讚嗎？有趣嗎？刺激嗎？</x:v>
+      </x:c>
+      <x:c r="F14" s="11" t="str">
+        <x:v>可以匿名嗎？可以刪掉嗎？可以轉傳嗎？</x:v>
+      </x:c>
+      <x:c r="G14" s="11" t="str">
         <x:v>是真的嗎？必要嗎？尊重嗎？</x:v>
       </x:c>
-      <x:c r="E14" s="11" t="str">
-        <x:v>夠快嗎？夠酸嗎？會紅嗎？</x:v>
-      </x:c>
-      <x:c r="F14" s="11" t="str">
-        <x:v>大家按讚嗎？有趣嗎？刺激嗎？</x:v>
-      </x:c>
-      <x:c r="G14" s="11" t="str">
-        <x:v>可以匿名嗎？可以刪掉嗎？可以轉傳嗎？</x:v>
-      </x:c>
       <x:c r="H14" s="11" t="n">
-        <x:v>13</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="I14" s="11" t="n">
         <x:v>30</x:v>
@@ -1514,16 +1514,16 @@
         <x:v>眼睛疲累</x:v>
       </x:c>
       <x:c r="E15" s="11" t="str">
+        <x:v>以上都可能</x:v>
+      </x:c>
+      <x:c r="F15" s="11" t="str">
         <x:v>睡不著</x:v>
       </x:c>
-      <x:c r="F15" s="11" t="str">
+      <x:c r="G15" s="11" t="str">
         <x:v>心情變差</x:v>
       </x:c>
-      <x:c r="G15" s="11" t="str">
-        <x:v>以上都可能</x:v>
-      </x:c>
       <x:c r="H15" s="11" t="n">
-        <x:v>14</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="I15" s="11" t="n">
         <x:v>30</x:v>
@@ -1555,7 +1555,7 @@
         <x:v>輸入帳號密碼確認</x:v>
       </x:c>
       <x:c r="H16" s="11" t="n">
-        <x:v>15</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I16" s="11" t="n">
         <x:v>30</x:v>
@@ -1581,13 +1581,13 @@
         <x:v>睡不好</x:v>
       </x:c>
       <x:c r="F17" s="11" t="str">
+        <x:v>以上都可能</x:v>
+      </x:c>
+      <x:c r="G17" s="11" t="str">
         <x:v>一直擔心來不及</x:v>
       </x:c>
-      <x:c r="G17" s="11" t="str">
-        <x:v>以上都可能</x:v>
-      </x:c>
       <x:c r="H17" s="11" t="n">
-        <x:v>16</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="I17" s="11" t="n">
         <x:v>30</x:v>
@@ -1607,19 +1607,19 @@
         <x:v>把焦慮轉成可執行的小目標。</x:v>
       </x:c>
       <x:c r="D18" s="11" t="str">
+        <x:v>永遠第一名</x:v>
+      </x:c>
+      <x:c r="E18" s="11" t="str">
+        <x:v>不要失敗</x:v>
+      </x:c>
+      <x:c r="F18" s="11" t="str">
+        <x:v>讓所有人都滿意</x:v>
+      </x:c>
+      <x:c r="G18" s="11" t="str">
         <x:v>今天完成 15 分鐘複習</x:v>
       </x:c>
-      <x:c r="E18" s="11" t="str">
-        <x:v>永遠第一名</x:v>
-      </x:c>
-      <x:c r="F18" s="11" t="str">
-        <x:v>不要失敗</x:v>
-      </x:c>
-      <x:c r="G18" s="11" t="str">
-        <x:v>讓所有人都滿意</x:v>
-      </x:c>
       <x:c r="H18" s="11" t="n">
-        <x:v>17</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="I18" s="11" t="n">
         <x:v>30</x:v>
@@ -1651,7 +1651,7 @@
         <x:v>算了，完全不要做</x:v>
       </x:c>
       <x:c r="H19" s="11" t="n">
-        <x:v>18</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I19" s="11" t="n">
         <x:v>30</x:v>
@@ -1671,10 +1671,10 @@
         <x:v>辨認安全且可信任的支持者。</x:v>
       </x:c>
       <x:c r="D20" s="11" t="str">
+        <x:v>只要求你忍耐的人</x:v>
+      </x:c>
+      <x:c r="E20" s="11" t="str">
         <x:v>願意聽、尊重界線並一起找方法的人</x:v>
-      </x:c>
-      <x:c r="E20" s="11" t="str">
-        <x:v>只要求你忍耐的人</x:v>
       </x:c>
       <x:c r="F20" s="11" t="str">
         <x:v>會把秘密公開的人</x:v>
@@ -1683,7 +1683,7 @@
         <x:v>完全不聽你說的人</x:v>
       </x:c>
       <x:c r="H20" s="11" t="n">
-        <x:v>19</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="I20" s="11" t="n">
         <x:v>30</x:v>
@@ -1709,13 +1709,13 @@
         <x:v>遇到困擾時找可信任的大人</x:v>
       </x:c>
       <x:c r="F21" s="11" t="str">
+        <x:v>以上都可以，選一個明天先試</x:v>
+      </x:c>
+      <x:c r="G21" s="11" t="str">
         <x:v>先查證再轉傳訊息</x:v>
       </x:c>
-      <x:c r="G21" s="11" t="str">
-        <x:v>以上都可以，選一個明天先試</x:v>
-      </x:c>
       <x:c r="H21" s="11" t="n">
-        <x:v>20</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="I21" s="11" t="n">
         <x:v>30</x:v>
@@ -1727,7 +1727,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R24e812f5d90b44d0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R012747be6ed240f2"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Use mixed Wayground question types
</commit_message>
<xml_diff>
--- a/xlsx/SEL平板暖身題庫_Wayground.xlsx
+++ b/xlsx/SEL平板暖身題庫_Wayground.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wayground匯入題庫" sheetId="1" r:id="Raff7737c0c1c44e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="教師備課對照" sheetId="2" r:id="R63e7fc4cbc554e6c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用說明" sheetId="3" r:id="R33820b08457d4353"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wayground匯入題庫" sheetId="1" r:id="R8e140a64ab24462a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="教師備課對照" sheetId="2" r:id="Rb98fdf4baee144ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用說明" sheetId="3" r:id="R596fc7ce9828486a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -413,24 +413,14 @@
         <x:v>如果今天的心情是一種天氣，你會選哪一種？</x:v>
       </x:c>
       <x:c r="B2" s="11" t="str">
-        <x:v>Multiple Choice</x:v>
-      </x:c>
-      <x:c r="C2" s="11" t="str">
-        <x:v>陰天</x:v>
-      </x:c>
-      <x:c r="D2" s="11" t="str">
-        <x:v>晴天</x:v>
-      </x:c>
-      <x:c r="E2" s="11" t="str">
-        <x:v>下雨</x:v>
-      </x:c>
-      <x:c r="F2" s="11" t="str">
-        <x:v>雷雨</x:v>
-      </x:c>
+        <x:v>Open-Ended</x:v>
+      </x:c>
+      <x:c r="C2" s="11" t="str"/>
+      <x:c r="D2" s="11" t="str"/>
+      <x:c r="E2" s="11" t="str"/>
+      <x:c r="F2" s="11" t="str"/>
       <x:c r="G2" s="11" t="str"/>
-      <x:c r="H2" s="11" t="n">
-        <x:v>2</x:v>
-      </x:c>
+      <x:c r="H2" s="11" t="str"/>
       <x:c r="I2" s="11" t="n">
         <x:v>30</x:v>
       </x:c>
@@ -506,7 +496,7 @@
         <x:v>當情緒溫度升到幾度時，可以先停一下再回應？</x:v>
       </x:c>
       <x:c r="B5" s="11" t="str">
-        <x:v>Multiple Choice</x:v>
+        <x:v>Poll</x:v>
       </x:c>
       <x:c r="C5" s="11" t="str">
         <x:v>沒有固定答案，察覺自己需要時就可以停</x:v>
@@ -521,9 +511,7 @@
         <x:v>3 度以上</x:v>
       </x:c>
       <x:c r="G5" s="11" t="str"/>
-      <x:c r="H5" s="11" t="n">
-        <x:v>1</x:v>
-      </x:c>
+      <x:c r="H5" s="11" t="str"/>
       <x:c r="I5" s="11" t="n">
         <x:v>30</x:v>
       </x:c>
@@ -661,24 +649,14 @@
         <x:v>小組裡有人一直沒有說話，你可以怎麼邀請？</x:v>
       </x:c>
       <x:c r="B10" s="11" t="str">
-        <x:v>Multiple Choice</x:v>
-      </x:c>
-      <x:c r="C10" s="11" t="str">
-        <x:v>你一定要現在回答</x:v>
-      </x:c>
-      <x:c r="D10" s="11" t="str">
-        <x:v>你想先聽聽他的想法嗎？也可以等一下再說</x:v>
-      </x:c>
-      <x:c r="E10" s="11" t="str">
-        <x:v>大家不要理他</x:v>
-      </x:c>
-      <x:c r="F10" s="11" t="str">
-        <x:v>替他直接決定</x:v>
-      </x:c>
+        <x:v>Open-Ended</x:v>
+      </x:c>
+      <x:c r="C10" s="11" t="str"/>
+      <x:c r="D10" s="11" t="str"/>
+      <x:c r="E10" s="11" t="str"/>
+      <x:c r="F10" s="11" t="str"/>
       <x:c r="G10" s="11" t="str"/>
-      <x:c r="H10" s="11" t="n">
-        <x:v>2</x:v>
-      </x:c>
+      <x:c r="H10" s="11" t="str"/>
       <x:c r="I10" s="11" t="n">
         <x:v>30</x:v>
       </x:c>
@@ -816,7 +794,7 @@
         <x:v>使用平板後，哪一個訊號提醒你需要休息？</x:v>
       </x:c>
       <x:c r="B15" s="11" t="str">
-        <x:v>Multiple Choice</x:v>
+        <x:v>Poll</x:v>
       </x:c>
       <x:c r="C15" s="11" t="str">
         <x:v>眼睛疲累</x:v>
@@ -831,9 +809,7 @@
         <x:v>心情變差</x:v>
       </x:c>
       <x:c r="G15" s="11" t="str"/>
-      <x:c r="H15" s="11" t="n">
-        <x:v>2</x:v>
-      </x:c>
+      <x:c r="H15" s="11" t="str"/>
       <x:c r="I15" s="11" t="n">
         <x:v>30</x:v>
       </x:c>
@@ -878,24 +854,14 @@
         <x:v>想到考試或升學時，哪一項可能是壓力訊號？</x:v>
       </x:c>
       <x:c r="B17" s="11" t="str">
-        <x:v>Multiple Choice</x:v>
-      </x:c>
-      <x:c r="C17" s="11" t="str">
-        <x:v>胃不舒服</x:v>
-      </x:c>
-      <x:c r="D17" s="11" t="str">
-        <x:v>睡不好</x:v>
-      </x:c>
-      <x:c r="E17" s="11" t="str">
-        <x:v>以上都可能</x:v>
-      </x:c>
-      <x:c r="F17" s="11" t="str">
-        <x:v>一直擔心來不及</x:v>
-      </x:c>
+        <x:v>Open-Ended</x:v>
+      </x:c>
+      <x:c r="C17" s="11" t="str"/>
+      <x:c r="D17" s="11" t="str"/>
+      <x:c r="E17" s="11" t="str"/>
+      <x:c r="F17" s="11" t="str"/>
       <x:c r="G17" s="11" t="str"/>
-      <x:c r="H17" s="11" t="n">
-        <x:v>3</x:v>
-      </x:c>
+      <x:c r="H17" s="11" t="str"/>
       <x:c r="I17" s="11" t="n">
         <x:v>30</x:v>
       </x:c>
@@ -940,24 +906,14 @@
         <x:v>把「我就是不行」改成哪一句支持自己的話？</x:v>
       </x:c>
       <x:c r="B19" s="11" t="str">
-        <x:v>Multiple Choice</x:v>
-      </x:c>
-      <x:c r="C19" s="11" t="str">
-        <x:v>我現在還不會，但我可以先試一小步</x:v>
-      </x:c>
-      <x:c r="D19" s="11" t="str">
-        <x:v>我永遠不可能學會</x:v>
-      </x:c>
-      <x:c r="E19" s="11" t="str">
-        <x:v>別人都比我好</x:v>
-      </x:c>
-      <x:c r="F19" s="11" t="str">
-        <x:v>算了，完全不要做</x:v>
-      </x:c>
+        <x:v>Open-Ended</x:v>
+      </x:c>
+      <x:c r="C19" s="11" t="str"/>
+      <x:c r="D19" s="11" t="str"/>
+      <x:c r="E19" s="11" t="str"/>
+      <x:c r="F19" s="11" t="str"/>
       <x:c r="G19" s="11" t="str"/>
-      <x:c r="H19" s="11" t="n">
-        <x:v>1</x:v>
-      </x:c>
+      <x:c r="H19" s="11" t="str"/>
       <x:c r="I19" s="11" t="n">
         <x:v>30</x:v>
       </x:c>
@@ -1002,7 +958,7 @@
         <x:v>課程結束後，你想把哪一個方法帶回生活？</x:v>
       </x:c>
       <x:c r="B21" s="11" t="str">
-        <x:v>Multiple Choice</x:v>
+        <x:v>Poll</x:v>
       </x:c>
       <x:c r="C21" s="11" t="str">
         <x:v>先辨認情緒和身體訊號</x:v>
@@ -1017,9 +973,7 @@
         <x:v>先查證再轉傳訊息</x:v>
       </x:c>
       <x:c r="G21" s="11" t="str"/>
-      <x:c r="H21" s="11" t="n">
-        <x:v>3</x:v>
-      </x:c>
+      <x:c r="H21" s="11" t="str"/>
       <x:c r="I21" s="11" t="n">
         <x:v>30</x:v>
       </x:c>
@@ -1031,7 +985,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra9d7b4976bac497c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb1d2b9f497304122"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1094,21 +1048,11 @@
       <x:c r="C2" s="11" t="str">
         <x:v>辨識當下情緒，不要求分享個人秘密。</x:v>
       </x:c>
-      <x:c r="D2" s="11" t="str">
-        <x:v>陰天</x:v>
-      </x:c>
-      <x:c r="E2" s="11" t="str">
-        <x:v>晴天</x:v>
-      </x:c>
-      <x:c r="F2" s="11" t="str">
-        <x:v>下雨</x:v>
-      </x:c>
-      <x:c r="G2" s="11" t="str">
-        <x:v>雷雨</x:v>
-      </x:c>
-      <x:c r="H2" s="11" t="n">
-        <x:v>2</x:v>
-      </x:c>
+      <x:c r="D2" s="11" t="str"/>
+      <x:c r="E2" s="11" t="str"/>
+      <x:c r="F2" s="11" t="str"/>
+      <x:c r="G2" s="11" t="str"/>
+      <x:c r="H2" s="11" t="str"/>
       <x:c r="I2" s="11" t="n">
         <x:v>30</x:v>
       </x:c>
@@ -1202,9 +1146,7 @@
       <x:c r="G5" s="11" t="str">
         <x:v>3 度以上</x:v>
       </x:c>
-      <x:c r="H5" s="11" t="n">
-        <x:v>1</x:v>
-      </x:c>
+      <x:c r="H5" s="11" t="str"/>
       <x:c r="I5" s="11" t="n">
         <x:v>30</x:v>
       </x:c>
@@ -1350,21 +1292,11 @@
       <x:c r="C10" s="11" t="str">
         <x:v>練習不強迫的團體邀請。</x:v>
       </x:c>
-      <x:c r="D10" s="11" t="str">
-        <x:v>你一定要現在回答</x:v>
-      </x:c>
-      <x:c r="E10" s="11" t="str">
-        <x:v>你想先聽聽他的想法嗎？也可以等一下再說</x:v>
-      </x:c>
-      <x:c r="F10" s="11" t="str">
-        <x:v>大家不要理他</x:v>
-      </x:c>
-      <x:c r="G10" s="11" t="str">
-        <x:v>替他直接決定</x:v>
-      </x:c>
-      <x:c r="H10" s="11" t="n">
-        <x:v>2</x:v>
-      </x:c>
+      <x:c r="D10" s="11" t="str"/>
+      <x:c r="E10" s="11" t="str"/>
+      <x:c r="F10" s="11" t="str"/>
+      <x:c r="G10" s="11" t="str"/>
+      <x:c r="H10" s="11" t="str"/>
       <x:c r="I10" s="11" t="n">
         <x:v>30</x:v>
       </x:c>
@@ -1522,9 +1454,7 @@
       <x:c r="G15" s="11" t="str">
         <x:v>心情變差</x:v>
       </x:c>
-      <x:c r="H15" s="11" t="n">
-        <x:v>2</x:v>
-      </x:c>
+      <x:c r="H15" s="11" t="str"/>
       <x:c r="I15" s="11" t="n">
         <x:v>30</x:v>
       </x:c>
@@ -1574,21 +1504,11 @@
       <x:c r="C17" s="11" t="str">
         <x:v>辨識升學與考試壓力的身心訊號。</x:v>
       </x:c>
-      <x:c r="D17" s="11" t="str">
-        <x:v>胃不舒服</x:v>
-      </x:c>
-      <x:c r="E17" s="11" t="str">
-        <x:v>睡不好</x:v>
-      </x:c>
-      <x:c r="F17" s="11" t="str">
-        <x:v>以上都可能</x:v>
-      </x:c>
-      <x:c r="G17" s="11" t="str">
-        <x:v>一直擔心來不及</x:v>
-      </x:c>
-      <x:c r="H17" s="11" t="n">
-        <x:v>3</x:v>
-      </x:c>
+      <x:c r="D17" s="11" t="str"/>
+      <x:c r="E17" s="11" t="str"/>
+      <x:c r="F17" s="11" t="str"/>
+      <x:c r="G17" s="11" t="str"/>
+      <x:c r="H17" s="11" t="str"/>
       <x:c r="I17" s="11" t="n">
         <x:v>30</x:v>
       </x:c>
@@ -1638,21 +1558,11 @@
       <x:c r="C19" s="11" t="str">
         <x:v>練習成長語句與自我支持。</x:v>
       </x:c>
-      <x:c r="D19" s="11" t="str">
-        <x:v>我現在還不會，但我可以先試一小步</x:v>
-      </x:c>
-      <x:c r="E19" s="11" t="str">
-        <x:v>我永遠不可能學會</x:v>
-      </x:c>
-      <x:c r="F19" s="11" t="str">
-        <x:v>別人都比我好</x:v>
-      </x:c>
-      <x:c r="G19" s="11" t="str">
-        <x:v>算了，完全不要做</x:v>
-      </x:c>
-      <x:c r="H19" s="11" t="n">
-        <x:v>1</x:v>
-      </x:c>
+      <x:c r="D19" s="11" t="str"/>
+      <x:c r="E19" s="11" t="str"/>
+      <x:c r="F19" s="11" t="str"/>
+      <x:c r="G19" s="11" t="str"/>
+      <x:c r="H19" s="11" t="str"/>
       <x:c r="I19" s="11" t="n">
         <x:v>30</x:v>
       </x:c>
@@ -1714,9 +1624,7 @@
       <x:c r="G21" s="11" t="str">
         <x:v>先查證再轉傳訊息</x:v>
       </x:c>
-      <x:c r="H21" s="11" t="n">
-        <x:v>3</x:v>
-      </x:c>
+      <x:c r="H21" s="11" t="str"/>
       <x:c r="I21" s="11" t="n">
         <x:v>30</x:v>
       </x:c>
@@ -1727,7 +1635,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R012747be6ed240f2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0cded633fa694126"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Update SEL teaching resources and notes
</commit_message>
<xml_diff>
--- a/xlsx/SEL平板暖身題庫_Wayground.xlsx
+++ b/xlsx/SEL平板暖身題庫_Wayground.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wayground匯入題庫" sheetId="1" r:id="R8e140a64ab24462a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="教師備課對照" sheetId="2" r:id="Rb98fdf4baee144ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用說明" sheetId="3" r:id="R596fc7ce9828486a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wayground匯入題庫" sheetId="1" r:id="R578464659e934821"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="教師備課對照" sheetId="2" r:id="R73d4de3d626b4ebf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用說明" sheetId="3" r:id="R1cfa5995821d4341"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -129,7 +129,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="WaygroundSELQuestionBank" displayName="WaygroundSELQuestionBank" ref="A1:K21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="WaygroundSELQuestionBank" displayName="WaygroundSELQuestionBank" ref="A1:K61" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Question Text"/>
     <x:tableColumn id="2" name="Question Type"/>
@@ -148,7 +148,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="SELTeacherNotes" displayName="SELTeacherNotes" ref="A1:J21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="SELTeacherNotes" displayName="SELTeacherNotes" ref="A1:J61" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="課次"/>
     <x:tableColumn id="2" name="暖身主題"/>
@@ -413,14 +413,24 @@
         <x:v>如果今天的心情是一種天氣，你會選哪一種？</x:v>
       </x:c>
       <x:c r="B2" s="11" t="str">
-        <x:v>Open-Ended</x:v>
-      </x:c>
-      <x:c r="C2" s="11" t="str"/>
-      <x:c r="D2" s="11" t="str"/>
-      <x:c r="E2" s="11" t="str"/>
-      <x:c r="F2" s="11" t="str"/>
+        <x:v>Multiple Choice</x:v>
+      </x:c>
+      <x:c r="C2" s="11" t="str">
+        <x:v>陰天</x:v>
+      </x:c>
+      <x:c r="D2" s="11" t="str">
+        <x:v>晴天</x:v>
+      </x:c>
+      <x:c r="E2" s="11" t="str">
+        <x:v>下雨</x:v>
+      </x:c>
+      <x:c r="F2" s="11" t="str">
+        <x:v>雷雨</x:v>
+      </x:c>
       <x:c r="G2" s="11" t="str"/>
-      <x:c r="H2" s="11" t="str"/>
+      <x:c r="H2" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="I2" s="11" t="n">
         <x:v>30</x:v>
       </x:c>
@@ -431,175 +441,177 @@
     </x:row>
     <x:row r="3" ht="78" customHeight="1">
       <x:c r="A3" s="10" t="str">
-        <x:v>當你緊張或煩躁時，哪一項可能是身體訊號？</x:v>
+        <x:v>描述心情時，哪一種說法最具體？</x:v>
       </x:c>
       <x:c r="B3" s="11" t="str">
         <x:v>Multiple Choice</x:v>
       </x:c>
       <x:c r="C3" s="11" t="str">
-        <x:v>心跳變快</x:v>
+        <x:v>我現在有點焦躁，肩膀也很緊</x:v>
       </x:c>
       <x:c r="D3" s="11" t="str">
-        <x:v>手心出汗</x:v>
+        <x:v>我沒事啦</x:v>
       </x:c>
       <x:c r="E3" s="11" t="str">
-        <x:v>肩膀變緊</x:v>
+        <x:v>大家都很煩</x:v>
       </x:c>
       <x:c r="F3" s="11" t="str">
-        <x:v>以上都可能</x:v>
+        <x:v>反正就是不好</x:v>
       </x:c>
       <x:c r="G3" s="11" t="str"/>
       <x:c r="H3" s="11" t="n">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I3" s="11" t="n">
         <x:v>30</x:v>
       </x:c>
       <x:c r="J3" s="11" t="str"/>
       <x:c r="K3" s="12" t="str">
-        <x:v>情緒常會先在身體出現訊號；察覺訊號能幫助我們提早停一下。</x:v>
+        <x:v>具體說出情緒和身體訊號，能幫助自己與他人理解目前需要。</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="78" customHeight="1">
       <x:c r="A4" s="10" t="str">
-        <x:v>同學突然身體不舒服時，哪一種做法最尊重？</x:v>
+        <x:v>當你還不確定自己的心情時，可以先做什麼？</x:v>
       </x:c>
       <x:c r="B4" s="11" t="str">
         <x:v>Multiple Choice</x:v>
       </x:c>
       <x:c r="C4" s="11" t="str">
-        <x:v>大聲詢問細節</x:v>
+        <x:v>立刻責怪自己</x:v>
       </x:c>
       <x:c r="D4" s="11" t="str">
-        <x:v>取笑對方</x:v>
+        <x:v>停一下，觀察身體和想法</x:v>
       </x:c>
       <x:c r="E4" s="11" t="str">
-        <x:v>安靜陪伴並通知可信任的大人</x:v>
+        <x:v>逼自己馬上說出答案</x:v>
       </x:c>
       <x:c r="F4" s="11" t="str">
-        <x:v>拍照傳到群組</x:v>
+        <x:v>假裝完全沒感覺</x:v>
       </x:c>
       <x:c r="G4" s="11" t="str"/>
       <x:c r="H4" s="11" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="I4" s="11" t="n">
         <x:v>30</x:v>
       </x:c>
       <x:c r="J4" s="11" t="str"/>
       <x:c r="K4" s="12" t="str">
-        <x:v>尊重包含保護隱私、提供陪伴，並在需要時找老師或校護協助。</x:v>
+        <x:v>不確定也沒關係，可以先停下來觀察，不必急著給自己貼標籤。</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="78" customHeight="1">
       <x:c r="A5" s="10" t="str">
-        <x:v>當情緒溫度升到幾度時，可以先停一下再回應？</x:v>
+        <x:v>當你緊張或煩躁時，哪一項可能是身體訊號？</x:v>
       </x:c>
       <x:c r="B5" s="11" t="str">
-        <x:v>Poll</x:v>
+        <x:v>Multiple Choice</x:v>
       </x:c>
       <x:c r="C5" s="11" t="str">
-        <x:v>沒有固定答案，察覺自己需要時就可以停</x:v>
+        <x:v>心跳變快</x:v>
       </x:c>
       <x:c r="D5" s="11" t="str">
-        <x:v>1 度</x:v>
+        <x:v>手心出汗</x:v>
       </x:c>
       <x:c r="E5" s="11" t="str">
-        <x:v>2 度</x:v>
+        <x:v>肩膀變緊</x:v>
       </x:c>
       <x:c r="F5" s="11" t="str">
-        <x:v>3 度以上</x:v>
+        <x:v>以上都可能</x:v>
       </x:c>
       <x:c r="G5" s="11" t="str"/>
-      <x:c r="H5" s="11" t="str"/>
+      <x:c r="H5" s="11" t="n">
+        <x:v>4</x:v>
+      </x:c>
       <x:c r="I5" s="11" t="n">
         <x:v>30</x:v>
       </x:c>
       <x:c r="J5" s="11" t="str"/>
       <x:c r="K5" s="12" t="str">
-        <x:v>每個人的警訊不同；當自己察覺快要失控或不舒服時，就可以先暫停。</x:v>
+        <x:v>情緒常會先在身體出現訊號；察覺訊號能幫助我們提早停一下。</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="78" customHeight="1">
       <x:c r="A6" s="10" t="str">
-        <x:v>遇到自己處理不了的困擾，第一個可以找誰？</x:v>
+        <x:v>下列哪一項也可能是緊張時的身體反應？</x:v>
       </x:c>
       <x:c r="B6" s="11" t="str">
         <x:v>Multiple Choice</x:v>
       </x:c>
       <x:c r="C6" s="11" t="str">
-        <x:v>完全不告訴任何人</x:v>
+        <x:v>突然長出翅膀</x:v>
       </x:c>
       <x:c r="D6" s="11" t="str">
-        <x:v>只在網路上找陌生人</x:v>
+        <x:v>完全不需要休息</x:v>
       </x:c>
       <x:c r="E6" s="11" t="str">
-        <x:v>責怪自己不夠勇敢</x:v>
+        <x:v>呼吸變快或變淺</x:v>
       </x:c>
       <x:c r="F6" s="11" t="str">
-        <x:v>可信任的導師、家人、校護或輔導老師</x:v>
+        <x:v>一定會發燒</x:v>
       </x:c>
       <x:c r="G6" s="11" t="str"/>
       <x:c r="H6" s="11" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="I6" s="11" t="n">
         <x:v>30</x:v>
       </x:c>
       <x:c r="J6" s="11" t="str"/>
       <x:c r="K6" s="12" t="str">
-        <x:v>求助可以從可信任的大人開始；遇到危險、受傷或持續困擾時，更要立即求助。</x:v>
+        <x:v>呼吸變快或變淺是常見的身體訊號，察覺後可以使用安全的調節方法。</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="78" customHeight="1">
       <x:c r="A7" s="10" t="str">
-        <x:v>朋友和你的喜好不一樣時，最好的第一步是什麼？</x:v>
+        <x:v>發現身體開始緊繃時，哪一個做法比較合適？</x:v>
       </x:c>
       <x:c r="B7" s="11" t="str">
         <x:v>Multiple Choice</x:v>
       </x:c>
       <x:c r="C7" s="11" t="str">
-        <x:v>逼對方改變</x:v>
+        <x:v>繼續硬撐到受不了</x:v>
       </x:c>
       <x:c r="D7" s="11" t="str">
-        <x:v>說出自己的喜好，也聽聽對方的想法</x:v>
+        <x:v>把責任推給別人</x:v>
       </x:c>
       <x:c r="E7" s="11" t="str">
-        <x:v>嘲笑對方</x:v>
+        <x:v>用傷害自己的方式發洩</x:v>
       </x:c>
       <x:c r="F7" s="11" t="str">
-        <x:v>假裝自己什麼都喜歡</x:v>
+        <x:v>先停下來，慢慢呼吸並觀察需要</x:v>
       </x:c>
       <x:c r="G7" s="11" t="str"/>
       <x:c r="H7" s="11" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="I7" s="11" t="n">
         <x:v>30</x:v>
       </x:c>
       <x:c r="J7" s="11" t="str"/>
       <x:c r="K7" s="12" t="str">
-        <x:v>友誼不必完全相同；表達自己並聽見對方，才有機會找到雙方都能接受的方式。</x:v>
+        <x:v>及早察覺並採取安全的暫停方式，有助於避免情緒繼續升高。</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="78" customHeight="1">
       <x:c r="A8" s="10" t="str">
-        <x:v>有人要求你分享不想分享的照片，你可以怎麼說？</x:v>
+        <x:v>同學突然身體不舒服時，哪一種做法最尊重？</x:v>
       </x:c>
       <x:c r="B8" s="11" t="str">
         <x:v>Multiple Choice</x:v>
       </x:c>
       <x:c r="C8" s="11" t="str">
-        <x:v>好啦，大家都傳了</x:v>
+        <x:v>大聲詢問細節</x:v>
       </x:c>
       <x:c r="D8" s="11" t="str">
-        <x:v>你不傳我就取笑你</x:v>
+        <x:v>取笑對方</x:v>
       </x:c>
       <x:c r="E8" s="11" t="str">
-        <x:v>我不想分享這張照片，請不要傳</x:v>
+        <x:v>安靜陪伴並通知可信任的大人</x:v>
       </x:c>
       <x:c r="F8" s="11" t="str">
-        <x:v>先傳給陌生人問問看</x:v>
+        <x:v>拍照傳到群組</x:v>
       </x:c>
       <x:c r="G8" s="11" t="str"/>
       <x:c r="H8" s="11" t="n">
@@ -610,27 +622,27 @@
       </x:c>
       <x:c r="J8" s="11" t="str"/>
       <x:c r="K8" s="12" t="str">
-        <x:v>清楚說不、停止轉傳並找可信任的大人，是保護自己和他人的做法。</x:v>
+        <x:v>尊重包含保護隱私、提供陪伴，並在需要時找老師或校護協助。</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="78" customHeight="1">
       <x:c r="A9" s="10" t="str">
-        <x:v>爭吵時，哪個動作能讓事情先停下來？</x:v>
+        <x:v>談到青春期身體變化時，哪一種態度較合適？</x:v>
       </x:c>
       <x:c r="B9" s="11" t="str">
         <x:v>Multiple Choice</x:v>
       </x:c>
       <x:c r="C9" s="11" t="str">
-        <x:v>深呼吸並暫時離開刺激</x:v>
+        <x:v>尊重差異，不拿別人的身體開玩笑</x:v>
       </x:c>
       <x:c r="D9" s="11" t="str">
-        <x:v>繼續大喊</x:v>
+        <x:v>比較誰變化最快</x:v>
       </x:c>
       <x:c r="E9" s="11" t="str">
-        <x:v>推人</x:v>
+        <x:v>替別人公開說明</x:v>
       </x:c>
       <x:c r="F9" s="11" t="str">
-        <x:v>立刻把爭吵內容轉傳</x:v>
+        <x:v>用綽號取笑對方</x:v>
       </x:c>
       <x:c r="G9" s="11" t="str"/>
       <x:c r="H9" s="11" t="n">
@@ -641,79 +653,89 @@
       </x:c>
       <x:c r="J9" s="11" t="str"/>
       <x:c r="K9" s="12" t="str">
-        <x:v>先讓身體降溫，才比較能說清楚、聽對方並找下一步；若有人害怕或受傷，要找大人。</x:v>
+        <x:v>每個人的成長速度不同，尊重隱私與差異是安全相處的重要原則。</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="78" customHeight="1">
       <x:c r="A10" s="10" t="str">
-        <x:v>小組裡有人一直沒有說話，你可以怎麼邀請？</x:v>
+        <x:v>同學需要衛生用品時，你可以怎麼協助？</x:v>
       </x:c>
       <x:c r="B10" s="11" t="str">
-        <x:v>Open-Ended</x:v>
-      </x:c>
-      <x:c r="C10" s="11" t="str"/>
-      <x:c r="D10" s="11" t="str"/>
-      <x:c r="E10" s="11" t="str"/>
-      <x:c r="F10" s="11" t="str"/>
+        <x:v>Multiple Choice</x:v>
+      </x:c>
+      <x:c r="C10" s="11" t="str">
+        <x:v>大聲問全班誰需要</x:v>
+      </x:c>
+      <x:c r="D10" s="11" t="str">
+        <x:v>低調提供資訊或陪同找可信任的大人</x:v>
+      </x:c>
+      <x:c r="E10" s="11" t="str">
+        <x:v>拍照記錄後分享</x:v>
+      </x:c>
+      <x:c r="F10" s="11" t="str">
+        <x:v>叫對方自己想辦法</x:v>
+      </x:c>
       <x:c r="G10" s="11" t="str"/>
-      <x:c r="H10" s="11" t="str"/>
+      <x:c r="H10" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="I10" s="11" t="n">
         <x:v>30</x:v>
       </x:c>
       <x:c r="J10" s="11" t="str"/>
       <x:c r="K10" s="12" t="str">
-        <x:v>好的邀請保留選擇，不強迫、不代替對方發言，讓每個人有安全參與的機會。</x:v>
+        <x:v>協助時要保護隱私，必要時陪同尋求老師、校護或其他可信任大人的支持。</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="78" customHeight="1">
       <x:c r="A11" s="10" t="str">
-        <x:v>面對朋友的請求，同意前需要先想什麼？</x:v>
+        <x:v>當情緒溫度升到幾度時，可以先停一下再回應？</x:v>
       </x:c>
       <x:c r="B11" s="11" t="str">
         <x:v>Multiple Choice</x:v>
       </x:c>
       <x:c r="C11" s="11" t="str">
-        <x:v>只要朋友開心就好</x:v>
+        <x:v>沒有固定答案，察覺自己需要時就可以停</x:v>
       </x:c>
       <x:c r="D11" s="11" t="str">
-        <x:v>別人怎麼做我就怎麼做</x:v>
+        <x:v>1 度</x:v>
       </x:c>
       <x:c r="E11" s="11" t="str">
-        <x:v>答應後再說</x:v>
+        <x:v>2 度</x:v>
       </x:c>
       <x:c r="F11" s="11" t="str">
-        <x:v>我的感受、我的界線和可能的結果</x:v>
+        <x:v>3 度以上</x:v>
       </x:c>
       <x:c r="G11" s="11" t="str"/>
       <x:c r="H11" s="11" t="n">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I11" s="11" t="n">
         <x:v>30</x:v>
       </x:c>
       <x:c r="J11" s="11" t="str"/>
       <x:c r="K11" s="12" t="str">
-        <x:v>負責任的決定要同時看見自己的感受、界線與可能結果，不必因為害怕失望而勉強自己。</x:v>
+        <x:v>每個人的警訊不同；當自己察覺快要失控或不舒服時，就可以先暫停。</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="78" customHeight="1">
       <x:c r="A12" s="10" t="str">
-        <x:v>看到「明天一定停課」的消息，你會先查哪一項？</x:v>
+        <x:v>情緒升高時，哪一個訊號表示你可能需要暫停？</x:v>
       </x:c>
       <x:c r="B12" s="11" t="str">
         <x:v>Multiple Choice</x:v>
       </x:c>
       <x:c r="C12" s="11" t="str">
-        <x:v>來源</x:v>
+        <x:v>覺得自己很平靜</x:v>
       </x:c>
       <x:c r="D12" s="11" t="str">
-        <x:v>日期</x:v>
+        <x:v>正在專心聽課</x:v>
       </x:c>
       <x:c r="E12" s="11" t="str">
-        <x:v>以上都要查</x:v>
+        <x:v>開始想大喊或做出衝動決定</x:v>
       </x:c>
       <x:c r="F12" s="11" t="str">
-        <x:v>證據</x:v>
+        <x:v>已經完成整理</x:v>
       </x:c>
       <x:c r="G12" s="11" t="str"/>
       <x:c r="H12" s="11" t="n">
@@ -724,58 +746,58 @@
       </x:c>
       <x:c r="J12" s="11" t="str"/>
       <x:c r="K12" s="12" t="str">
-        <x:v>查證時可以看來源、日期、證據與發布目的，再和可信來源比對，不急著轉傳。</x:v>
+        <x:v>衝動感變強是可以提醒自己先暫停的訊號，不必等到事情失控才處理。</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="78" customHeight="1">
       <x:c r="A13" s="10" t="str">
-        <x:v>下列哪一項不適合提供給陌生帳號？</x:v>
+        <x:v>安全暫停後，回到對話前可以先做什麼？</x:v>
       </x:c>
       <x:c r="B13" s="11" t="str">
         <x:v>Multiple Choice</x:v>
       </x:c>
       <x:c r="C13" s="11" t="str">
-        <x:v>住址</x:v>
+        <x:v>立刻回去爭輸贏</x:v>
       </x:c>
       <x:c r="D13" s="11" t="str">
-        <x:v>喜歡的顏色</x:v>
+        <x:v>把對方的話公開</x:v>
       </x:c>
       <x:c r="E13" s="11" t="str">
-        <x:v>喜歡的遊戲角色</x:v>
+        <x:v>完全不必理會任何人</x:v>
       </x:c>
       <x:c r="F13" s="11" t="str">
-        <x:v>喜歡的食物</x:v>
+        <x:v>確認自己已比較穩定，再選擇說法或求助</x:v>
       </x:c>
       <x:c r="G13" s="11" t="str"/>
       <x:c r="H13" s="11" t="n">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="I13" s="11" t="n">
         <x:v>30</x:v>
       </x:c>
       <x:c r="J13" s="11" t="str"/>
       <x:c r="K13" s="12" t="str">
-        <x:v>住址屬於個人資料，不應提供給陌生帳號；遇到索取或威脅，截圖、封鎖並告訴大人。</x:v>
+        <x:v>暫停的目的是恢復選擇能力，穩定後再決定要溝通、離開或找大人。</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="78" customHeight="1">
       <x:c r="A14" s="10" t="str">
-        <x:v>留言送出前，可以用哪三個問題檢查？</x:v>
+        <x:v>遇到自己處理不了的困擾，第一個可以找誰？</x:v>
       </x:c>
       <x:c r="B14" s="11" t="str">
         <x:v>Multiple Choice</x:v>
       </x:c>
       <x:c r="C14" s="11" t="str">
-        <x:v>夠快嗎？夠酸嗎？會紅嗎？</x:v>
+        <x:v>完全不告訴任何人</x:v>
       </x:c>
       <x:c r="D14" s="11" t="str">
-        <x:v>大家按讚嗎？有趣嗎？刺激嗎？</x:v>
+        <x:v>只在網路上找陌生人</x:v>
       </x:c>
       <x:c r="E14" s="11" t="str">
-        <x:v>可以匿名嗎？可以刪掉嗎？可以轉傳嗎？</x:v>
+        <x:v>責怪自己不夠勇敢</x:v>
       </x:c>
       <x:c r="F14" s="11" t="str">
-        <x:v>是真的嗎？必要嗎？尊重嗎？</x:v>
+        <x:v>可信任的導師、家人、校護或輔導老師</x:v>
       </x:c>
       <x:c r="G14" s="11" t="str"/>
       <x:c r="H14" s="11" t="n">
@@ -786,206 +808,1470 @@
       </x:c>
       <x:c r="J14" s="11" t="str"/>
       <x:c r="K14" s="12" t="str">
-        <x:v>留言前三問能幫助我們降低誤會與傷害：內容是否真實、是否必要、是否尊重。</x:v>
+        <x:v>求助可以從可信任的大人開始；遇到危險、受傷或持續困擾時，更要立即求助。</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="78" customHeight="1">
       <x:c r="A15" s="10" t="str">
-        <x:v>使用平板後，哪一個訊號提醒你需要休息？</x:v>
+        <x:v>求助時，怎麼描述事情比較有幫助？</x:v>
       </x:c>
       <x:c r="B15" s="11" t="str">
-        <x:v>Poll</x:v>
+        <x:v>Multiple Choice</x:v>
       </x:c>
       <x:c r="C15" s="11" t="str">
-        <x:v>眼睛疲累</x:v>
+        <x:v>說明發生什麼、何時發生，以及自己需要什麼</x:v>
       </x:c>
       <x:c r="D15" s="11" t="str">
-        <x:v>以上都可能</x:v>
+        <x:v>只說「你自己猜」</x:v>
       </x:c>
       <x:c r="E15" s="11" t="str">
-        <x:v>睡不著</x:v>
+        <x:v>先責怪自己</x:v>
       </x:c>
       <x:c r="F15" s="11" t="str">
-        <x:v>心情變差</x:v>
+        <x:v>完全不提供線索</x:v>
       </x:c>
       <x:c r="G15" s="11" t="str"/>
-      <x:c r="H15" s="11" t="str"/>
+      <x:c r="H15" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="I15" s="11" t="n">
         <x:v>30</x:v>
       </x:c>
       <x:c r="J15" s="11" t="str"/>
       <x:c r="K15" s="12" t="str">
-        <x:v>身體和情緒訊號都值得注意；可以關閉通知、固定休息，並安排不使用螢幕的替代活動。</x:v>
+        <x:v>清楚描述事件、時間與需要，能幫助可信任的大人更快理解並提供協助。</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="78" customHeight="1">
       <x:c r="A16" s="10" t="str">
-        <x:v>遇到可疑連結，第一步應該做什麼？</x:v>
+        <x:v>如果第一位大人沒有立即回應，你可以怎麼辦？</x:v>
       </x:c>
       <x:c r="B16" s="11" t="str">
         <x:v>Multiple Choice</x:v>
       </x:c>
       <x:c r="C16" s="11" t="str">
-        <x:v>先停下來，不點開、不輸入資料</x:v>
+        <x:v>就此放棄</x:v>
       </x:c>
       <x:c r="D16" s="11" t="str">
-        <x:v>好奇地點開看看</x:v>
+        <x:v>再找另一位可信任的大人，持續求助</x:v>
       </x:c>
       <x:c r="E16" s="11" t="str">
-        <x:v>轉傳給同學測試</x:v>
+        <x:v>把事情傳給陌生人</x:v>
       </x:c>
       <x:c r="F16" s="11" t="str">
-        <x:v>輸入帳號密碼確認</x:v>
+        <x:v>責怪自己不值得幫忙</x:v>
       </x:c>
       <x:c r="G16" s="11" t="str"/>
       <x:c r="H16" s="11" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="I16" s="11" t="n">
         <x:v>30</x:v>
       </x:c>
       <x:c r="J16" s="11" t="str"/>
       <x:c r="K16" s="12" t="str">
-        <x:v>可疑連結先不點、不輸入資料，保留訊息並找可信任的大人或正式管道確認。</x:v>
+        <x:v>找不到合適的回應時可以繼續找其他可信任的大人，安全與需要被看見很重要。</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="78" customHeight="1">
       <x:c r="A17" s="10" t="str">
-        <x:v>想到考試或升學時，哪一項可能是壓力訊號？</x:v>
+        <x:v>朋友和你的喜好不一樣時，最好的第一步是什麼？</x:v>
       </x:c>
       <x:c r="B17" s="11" t="str">
-        <x:v>Open-Ended</x:v>
-      </x:c>
-      <x:c r="C17" s="11" t="str"/>
-      <x:c r="D17" s="11" t="str"/>
-      <x:c r="E17" s="11" t="str"/>
-      <x:c r="F17" s="11" t="str"/>
+        <x:v>Multiple Choice</x:v>
+      </x:c>
+      <x:c r="C17" s="11" t="str">
+        <x:v>逼對方改變</x:v>
+      </x:c>
+      <x:c r="D17" s="11" t="str">
+        <x:v>說出自己的喜好，也聽聽對方的想法</x:v>
+      </x:c>
+      <x:c r="E17" s="11" t="str">
+        <x:v>嘲笑對方</x:v>
+      </x:c>
+      <x:c r="F17" s="11" t="str">
+        <x:v>假裝自己什麼都喜歡</x:v>
+      </x:c>
       <x:c r="G17" s="11" t="str"/>
-      <x:c r="H17" s="11" t="str"/>
+      <x:c r="H17" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="I17" s="11" t="n">
         <x:v>30</x:v>
       </x:c>
       <x:c r="J17" s="11" t="str"/>
       <x:c r="K17" s="12" t="str">
-        <x:v>壓力可能同時出現在身體、睡眠和想法；先辨認訊號，再把事情分成可控制與暫時不可控制。</x:v>
+        <x:v>友誼不必完全相同；表達自己並聽見對方，才有機會找到雙方都能接受的方式。</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="78" customHeight="1">
       <x:c r="A18" s="10" t="str">
-        <x:v>「我要變厲害」可以改成哪一種比較可行的目標？</x:v>
+        <x:v>朋友意見不同時，哪一句話有助於保持尊重？</x:v>
       </x:c>
       <x:c r="B18" s="11" t="str">
         <x:v>Multiple Choice</x:v>
       </x:c>
       <x:c r="C18" s="11" t="str">
-        <x:v>永遠第一名</x:v>
+        <x:v>你怎麼這麼笨</x:v>
       </x:c>
       <x:c r="D18" s="11" t="str">
-        <x:v>不要失敗</x:v>
+        <x:v>你一定要照我的</x:v>
       </x:c>
       <x:c r="E18" s="11" t="str">
-        <x:v>讓所有人都滿意</x:v>
+        <x:v>我和你想法不同，但我們可以聽聽彼此</x:v>
       </x:c>
       <x:c r="F18" s="11" t="str">
-        <x:v>今天完成 15 分鐘複習</x:v>
+        <x:v>那就不要再當朋友</x:v>
       </x:c>
       <x:c r="G18" s="11" t="str"/>
       <x:c r="H18" s="11" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="I18" s="11" t="n">
         <x:v>30</x:v>
       </x:c>
       <x:c r="J18" s="11" t="str"/>
       <x:c r="K18" s="12" t="str">
-        <x:v>可行目標要具體、能在近期開始；把大目標拆成今天的一小步，較容易看見進展。</x:v>
+        <x:v>表達差異並願意聆聽，可以讓關係保留合作與選擇的空間。</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="78" customHeight="1">
       <x:c r="A19" s="10" t="str">
-        <x:v>把「我就是不行」改成哪一句支持自己的話？</x:v>
+        <x:v>和朋友安排活動時，怎麼做比較公平？</x:v>
       </x:c>
       <x:c r="B19" s="11" t="str">
-        <x:v>Open-Ended</x:v>
-      </x:c>
-      <x:c r="C19" s="11" t="str"/>
-      <x:c r="D19" s="11" t="str"/>
-      <x:c r="E19" s="11" t="str"/>
-      <x:c r="F19" s="11" t="str"/>
+        <x:v>Multiple Choice</x:v>
+      </x:c>
+      <x:c r="C19" s="11" t="str">
+        <x:v>永遠只聽一個人的</x:v>
+      </x:c>
+      <x:c r="D19" s="11" t="str">
+        <x:v>誰大聲誰決定</x:v>
+      </x:c>
+      <x:c r="E19" s="11" t="str">
+        <x:v>完全不討論</x:v>
+      </x:c>
+      <x:c r="F19" s="11" t="str">
+        <x:v>輪流選擇，或一起找雙方都能接受的方案</x:v>
+      </x:c>
       <x:c r="G19" s="11" t="str"/>
-      <x:c r="H19" s="11" t="str"/>
+      <x:c r="H19" s="11" t="n">
+        <x:v>4</x:v>
+      </x:c>
       <x:c r="I19" s="11" t="n">
         <x:v>30</x:v>
       </x:c>
       <x:c r="J19" s="11" t="str"/>
       <x:c r="K19" s="12" t="str">
-        <x:v>成長語句不否認困難，而是把注意力放回目前能學習或嘗試的下一步。</x:v>
+        <x:v>輪流與協商能讓彼此的需要被看見，也不必要求喜好完全相同。</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="78" customHeight="1">
       <x:c r="A20" s="10" t="str">
-        <x:v>遇到壓力時，什麼樣的大人可以成為支持者？</x:v>
+        <x:v>有人要求你分享不想分享的照片，你可以怎麼說？</x:v>
       </x:c>
       <x:c r="B20" s="11" t="str">
         <x:v>Multiple Choice</x:v>
       </x:c>
       <x:c r="C20" s="11" t="str">
-        <x:v>只要求你忍耐的人</x:v>
+        <x:v>好啦，大家都傳了</x:v>
       </x:c>
       <x:c r="D20" s="11" t="str">
-        <x:v>願意聽、尊重界線並一起找方法的人</x:v>
+        <x:v>你不傳我就取笑你</x:v>
       </x:c>
       <x:c r="E20" s="11" t="str">
-        <x:v>會把秘密公開的人</x:v>
+        <x:v>我不想分享這張照片，請不要傳</x:v>
       </x:c>
       <x:c r="F20" s="11" t="str">
-        <x:v>完全不聽你說的人</x:v>
+        <x:v>先傳給陌生人問問看</x:v>
       </x:c>
       <x:c r="G20" s="11" t="str"/>
       <x:c r="H20" s="11" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="I20" s="11" t="n">
         <x:v>30</x:v>
       </x:c>
       <x:c r="J20" s="11" t="str"/>
       <x:c r="K20" s="12" t="str">
-        <x:v>支持者不一定直接替你解決，但會願意聽、尊重界線，必要時陪你找合適的協助。</x:v>
+        <x:v>清楚說不、停止轉傳並找可信任的大人，是保護自己和他人的做法。</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="78" customHeight="1">
       <x:c r="A21" s="10" t="str">
-        <x:v>課程結束後，你想把哪一個方法帶回生活？</x:v>
+        <x:v>別人傳來你的照片並要求你不要告訴大人，你可以怎麼做？</x:v>
       </x:c>
       <x:c r="B21" s="11" t="str">
-        <x:v>Poll</x:v>
+        <x:v>Multiple Choice</x:v>
       </x:c>
       <x:c r="C21" s="11" t="str">
-        <x:v>先辨認情緒和身體訊號</x:v>
+        <x:v>保留訊息、停止轉傳並找可信任的大人</x:v>
       </x:c>
       <x:c r="D21" s="11" t="str">
-        <x:v>遇到困擾時找可信任的大人</x:v>
+        <x:v>照對方要求保守秘密</x:v>
       </x:c>
       <x:c r="E21" s="11" t="str">
-        <x:v>以上都可以，選一個明天先試</x:v>
+        <x:v>再轉給更多人</x:v>
       </x:c>
       <x:c r="F21" s="11" t="str">
-        <x:v>先查證再轉傳訊息</x:v>
+        <x:v>刪除所有證據後忍耐</x:v>
       </x:c>
       <x:c r="G21" s="11" t="str"/>
-      <x:c r="H21" s="11" t="str"/>
+      <x:c r="H21" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="I21" s="11" t="n">
         <x:v>30</x:v>
       </x:c>
       <x:c r="J21" s="11" t="str"/>
       <x:c r="K21" s="12" t="str">
+        <x:v>遇到不舒服或被威脅的影像情境，保留紀錄、停止轉傳並求助能增加安全。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="78" customHeight="1">
+      <x:c r="A22" s="10" t="str">
+        <x:v>拒絕別人的要求時，哪一句最清楚？</x:v>
+      </x:c>
+      <x:c r="B22" s="11" t="str">
+        <x:v>Multiple Choice</x:v>
+      </x:c>
+      <x:c r="C22" s="11" t="str">
+        <x:v>你應該知道我不想要</x:v>
+      </x:c>
+      <x:c r="D22" s="11" t="str">
+        <x:v>我不願意，請停止；需要時我會找大人</x:v>
+      </x:c>
+      <x:c r="E22" s="11" t="str">
+        <x:v>隨便你啦</x:v>
+      </x:c>
+      <x:c r="F22" s="11" t="str">
+        <x:v>我先答應再後悔</x:v>
+      </x:c>
+      <x:c r="G22" s="11" t="str"/>
+      <x:c r="H22" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I22" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J22" s="11" t="str"/>
+      <x:c r="K22" s="12" t="str">
+        <x:v>清楚說明不願意和下一步，能幫助自己守住界線並尋求支持。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="78" customHeight="1">
+      <x:c r="A23" s="10" t="str">
+        <x:v>爭吵時，哪個動作能讓事情先停下來？</x:v>
+      </x:c>
+      <x:c r="B23" s="11" t="str">
+        <x:v>Multiple Choice</x:v>
+      </x:c>
+      <x:c r="C23" s="11" t="str">
+        <x:v>深呼吸並暫時離開刺激</x:v>
+      </x:c>
+      <x:c r="D23" s="11" t="str">
+        <x:v>繼續大喊</x:v>
+      </x:c>
+      <x:c r="E23" s="11" t="str">
+        <x:v>推人</x:v>
+      </x:c>
+      <x:c r="F23" s="11" t="str">
+        <x:v>立刻把爭吵內容轉傳</x:v>
+      </x:c>
+      <x:c r="G23" s="11" t="str"/>
+      <x:c r="H23" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I23" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J23" s="11" t="str"/>
+      <x:c r="K23" s="12" t="str">
+        <x:v>先讓身體降溫，才比較能說清楚、聽對方並找下一步；若有人害怕或受傷，要找大人。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="78" customHeight="1">
+      <x:c r="A24" s="10" t="str">
+        <x:v>衝突中想回應前，哪一個做法能增加安全？</x:v>
+      </x:c>
+      <x:c r="B24" s="11" t="str">
+        <x:v>Multiple Choice</x:v>
+      </x:c>
+      <x:c r="C24" s="11" t="str">
+        <x:v>靠近對方繼續挑釁</x:v>
+      </x:c>
+      <x:c r="D24" s="11" t="str">
+        <x:v>立刻錄影上傳</x:v>
+      </x:c>
+      <x:c r="E24" s="11" t="str">
+        <x:v>先確認自己與他人都沒有受傷，再決定是否對話</x:v>
+      </x:c>
+      <x:c r="F24" s="11" t="str">
+        <x:v>用力推開對方</x:v>
+      </x:c>
+      <x:c r="G24" s="11" t="str"/>
+      <x:c r="H24" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I24" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J24" s="11" t="str"/>
+      <x:c r="K24" s="12" t="str">
+        <x:v>先確認安全，再決定暫停、離開或找大人，優先保護自己與他人。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="78" customHeight="1">
+      <x:c r="A25" s="10" t="str">
+        <x:v>衝突後想修復關係，可以先說什麼？</x:v>
+      </x:c>
+      <x:c r="B25" s="11" t="str">
+        <x:v>Multiple Choice</x:v>
+      </x:c>
+      <x:c r="C25" s="11" t="str">
+        <x:v>都是你害的</x:v>
+      </x:c>
+      <x:c r="D25" s="11" t="str">
+        <x:v>你不准再提</x:v>
+      </x:c>
+      <x:c r="E25" s="11" t="str">
+        <x:v>我道歉但你不能有意見</x:v>
+      </x:c>
+      <x:c r="F25" s="11" t="str">
+        <x:v>我剛才的做法讓你不舒服，我想聽聽你的感受</x:v>
+      </x:c>
+      <x:c r="G25" s="11" t="str"/>
+      <x:c r="H25" s="11" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I25" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J25" s="11" t="str"/>
+      <x:c r="K25" s="12" t="str">
+        <x:v>修復包含承認影響、聆聽感受與一起討論下一步，不是逼對方立刻原諒。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="78" customHeight="1">
+      <x:c r="A26" s="10" t="str">
+        <x:v>小組裡有人一直沒有說話，你可以怎麼邀請？</x:v>
+      </x:c>
+      <x:c r="B26" s="11" t="str">
+        <x:v>Multiple Choice</x:v>
+      </x:c>
+      <x:c r="C26" s="11" t="str">
+        <x:v>你一定要現在回答</x:v>
+      </x:c>
+      <x:c r="D26" s="11" t="str">
+        <x:v>你想先聽聽他的想法嗎？也可以等一下再說</x:v>
+      </x:c>
+      <x:c r="E26" s="11" t="str">
+        <x:v>大家不要理他</x:v>
+      </x:c>
+      <x:c r="F26" s="11" t="str">
+        <x:v>替他直接決定</x:v>
+      </x:c>
+      <x:c r="G26" s="11" t="str"/>
+      <x:c r="H26" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I26" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J26" s="11" t="str"/>
+      <x:c r="K26" s="12" t="str">
+        <x:v>好的邀請保留選擇，不強迫、不代替對方發言，讓每個人有安全參與的機會。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="78" customHeight="1">
+      <x:c r="A27" s="10" t="str">
+        <x:v>邀請小組成員發言時，哪一種做法最有選擇？</x:v>
+      </x:c>
+      <x:c r="B27" s="11" t="str">
+        <x:v>Multiple Choice</x:v>
+      </x:c>
+      <x:c r="C27" s="11" t="str">
+        <x:v>你想現在說，還是先用寫的？</x:v>
+      </x:c>
+      <x:c r="D27" s="11" t="str">
+        <x:v>你一定要說</x:v>
+      </x:c>
+      <x:c r="E27" s="11" t="str">
+        <x:v>不說就扣分</x:v>
+      </x:c>
+      <x:c r="F27" s="11" t="str">
+        <x:v>我替你回答</x:v>
+      </x:c>
+      <x:c r="G27" s="11" t="str"/>
+      <x:c r="H27" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I27" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J27" s="11" t="str"/>
+      <x:c r="K27" s="12" t="str">
+        <x:v>提供不同參與方式能降低壓力，也尊重每個人的準備時間與界線。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="78" customHeight="1">
+      <x:c r="A28" s="10" t="str">
+        <x:v>小組合作時，如何讓安靜的同學也有參與機會？</x:v>
+      </x:c>
+      <x:c r="B28" s="11" t="str">
+        <x:v>Multiple Choice</x:v>
+      </x:c>
+      <x:c r="C28" s="11" t="str">
+        <x:v>直接替他決定全部工作</x:v>
+      </x:c>
+      <x:c r="D28" s="11" t="str">
+        <x:v>先詢問意願，再安排適合的角色</x:v>
+      </x:c>
+      <x:c r="E28" s="11" t="str">
+        <x:v>要求他代表全組發言</x:v>
+      </x:c>
+      <x:c r="F28" s="11" t="str">
+        <x:v>完全忽略他的想法</x:v>
+      </x:c>
+      <x:c r="G28" s="11" t="str"/>
+      <x:c r="H28" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I28" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J28" s="11" t="str"/>
+      <x:c r="K28" s="12" t="str">
+        <x:v>先詢問意願並提供角色選擇，能讓參與更安全也更公平。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="78" customHeight="1">
+      <x:c r="A29" s="10" t="str">
+        <x:v>面對朋友的請求，同意前需要先想什麼？</x:v>
+      </x:c>
+      <x:c r="B29" s="11" t="str">
+        <x:v>Multiple Choice</x:v>
+      </x:c>
+      <x:c r="C29" s="11" t="str">
+        <x:v>只要朋友開心就好</x:v>
+      </x:c>
+      <x:c r="D29" s="11" t="str">
+        <x:v>別人怎麼做我就怎麼做</x:v>
+      </x:c>
+      <x:c r="E29" s="11" t="str">
+        <x:v>答應後再說</x:v>
+      </x:c>
+      <x:c r="F29" s="11" t="str">
+        <x:v>我的感受、我的界線和可能的結果</x:v>
+      </x:c>
+      <x:c r="G29" s="11" t="str"/>
+      <x:c r="H29" s="11" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I29" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J29" s="11" t="str"/>
+      <x:c r="K29" s="12" t="str">
+        <x:v>負責任的決定要同時看見自己的感受、界線與可能結果，不必因為害怕失望而勉強自己。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="78" customHeight="1">
+      <x:c r="A30" s="10" t="str">
+        <x:v>需要拒絕朋友時，哪一種順序比較清楚？</x:v>
+      </x:c>
+      <x:c r="B30" s="11" t="str">
+        <x:v>Multiple Choice</x:v>
+      </x:c>
+      <x:c r="C30" s="11" t="str">
+        <x:v>先答應再想辦法</x:v>
+      </x:c>
+      <x:c r="D30" s="11" t="str">
+        <x:v>先嘲笑對方</x:v>
+      </x:c>
+      <x:c r="E30" s="11" t="str">
+        <x:v>先說感受或界線，再說可以接受的替代方案</x:v>
+      </x:c>
+      <x:c r="F30" s="11" t="str">
+        <x:v>完全不回應</x:v>
+      </x:c>
+      <x:c r="G30" s="11" t="str"/>
+      <x:c r="H30" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I30" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J30" s="11" t="str"/>
+      <x:c r="K30" s="12" t="str">
+        <x:v>先表達界線，再提出替代方案，有助於兼顧自己需要與關係溝通。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="78" customHeight="1">
+      <x:c r="A31" s="10" t="str">
+        <x:v>做決定前，哪一個問題最值得先問自己？</x:v>
+      </x:c>
+      <x:c r="B31" s="11" t="str">
+        <x:v>Multiple Choice</x:v>
+      </x:c>
+      <x:c r="C31" s="11" t="str">
+        <x:v>大家會不會都稱讚我？</x:v>
+      </x:c>
+      <x:c r="D31" s="11" t="str">
+        <x:v>最快可以結束嗎？</x:v>
+      </x:c>
+      <x:c r="E31" s="11" t="str">
+        <x:v>別人是否都這樣做？</x:v>
+      </x:c>
+      <x:c r="F31" s="11" t="str">
+        <x:v>這符合我的感受與界線嗎？</x:v>
+      </x:c>
+      <x:c r="G31" s="11" t="str"/>
+      <x:c r="H31" s="11" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I31" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J31" s="11" t="str"/>
+      <x:c r="K31" s="12" t="str">
+        <x:v>把自己的感受、界線和可能結果放進決定中，能減少因壓力而勉強自己。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="78" customHeight="1">
+      <x:c r="A32" s="10" t="str">
+        <x:v>看到「明天一定停課」的消息，你會先查哪一項？</x:v>
+      </x:c>
+      <x:c r="B32" s="11" t="str">
+        <x:v>Multiple Choice</x:v>
+      </x:c>
+      <x:c r="C32" s="11" t="str">
+        <x:v>來源</x:v>
+      </x:c>
+      <x:c r="D32" s="11" t="str">
+        <x:v>日期</x:v>
+      </x:c>
+      <x:c r="E32" s="11" t="str">
+        <x:v>以上都要查</x:v>
+      </x:c>
+      <x:c r="F32" s="11" t="str">
+        <x:v>證據</x:v>
+      </x:c>
+      <x:c r="G32" s="11" t="str"/>
+      <x:c r="H32" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I32" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J32" s="11" t="str"/>
+      <x:c r="K32" s="12" t="str">
+        <x:v>查證時可以看來源、日期、證據與發布目的，再和可信來源比對，不急著轉傳。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="78" customHeight="1">
+      <x:c r="A33" s="10" t="str">
+        <x:v>查證網路消息時，哪一項線索最需要留意？</x:v>
+      </x:c>
+      <x:c r="B33" s="11" t="str">
+        <x:v>Multiple Choice</x:v>
+      </x:c>
+      <x:c r="C33" s="11" t="str">
+        <x:v>發布者是否可信、內容是否有日期與證據</x:v>
+      </x:c>
+      <x:c r="D33" s="11" t="str">
+        <x:v>標題是否夠生氣</x:v>
+      </x:c>
+      <x:c r="E33" s="11" t="str">
+        <x:v>轉發人數是否很多</x:v>
+      </x:c>
+      <x:c r="F33" s="11" t="str">
+        <x:v>圖片是否夠吸睛</x:v>
+      </x:c>
+      <x:c r="G33" s="11" t="str"/>
+      <x:c r="H33" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I33" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J33" s="11" t="str"/>
+      <x:c r="K33" s="12" t="str">
+        <x:v>可信來源、日期與證據，比情緒化標題或轉發數更能幫助判斷訊息。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="78" customHeight="1">
+      <x:c r="A34" s="10" t="str">
+        <x:v>看到不確定的消息時，最負責任的做法是什麼？</x:v>
+      </x:c>
+      <x:c r="B34" s="11" t="str">
+        <x:v>Multiple Choice</x:v>
+      </x:c>
+      <x:c r="C34" s="11" t="str">
+        <x:v>先轉傳再說</x:v>
+      </x:c>
+      <x:c r="D34" s="11" t="str">
+        <x:v>先暫停轉傳，查到可信資料再決定</x:v>
+      </x:c>
+      <x:c r="E34" s="11" t="str">
+        <x:v>只看留言猜測</x:v>
+      </x:c>
+      <x:c r="F34" s="11" t="str">
+        <x:v>把疑問改成肯定語氣</x:v>
+      </x:c>
+      <x:c r="G34" s="11" t="str"/>
+      <x:c r="H34" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I34" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J34" s="11" t="str"/>
+      <x:c r="K34" s="12" t="str">
+        <x:v>不急著轉傳能降低錯誤訊息擴散，也保留查證與修正的空間。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="78" customHeight="1">
+      <x:c r="A35" s="10" t="str">
+        <x:v>下列哪一項不適合提供給陌生帳號？</x:v>
+      </x:c>
+      <x:c r="B35" s="11" t="str">
+        <x:v>Multiple Choice</x:v>
+      </x:c>
+      <x:c r="C35" s="11" t="str">
+        <x:v>住址</x:v>
+      </x:c>
+      <x:c r="D35" s="11" t="str">
+        <x:v>喜歡的顏色</x:v>
+      </x:c>
+      <x:c r="E35" s="11" t="str">
+        <x:v>喜歡的遊戲角色</x:v>
+      </x:c>
+      <x:c r="F35" s="11" t="str">
+        <x:v>喜歡的食物</x:v>
+      </x:c>
+      <x:c r="G35" s="11" t="str"/>
+      <x:c r="H35" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I35" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J35" s="11" t="str"/>
+      <x:c r="K35" s="12" t="str">
+        <x:v>住址屬於個人資料，不應提供給陌生帳號；遇到索取或威脅，截圖、封鎖並告訴大人。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="78" customHeight="1">
+      <x:c r="A36" s="10" t="str">
+        <x:v>下列哪一項屬於個人資料，需要謹慎保護？</x:v>
+      </x:c>
+      <x:c r="B36" s="11" t="str">
+        <x:v>Multiple Choice</x:v>
+      </x:c>
+      <x:c r="C36" s="11" t="str">
+        <x:v>喜歡的顏色</x:v>
+      </x:c>
+      <x:c r="D36" s="11" t="str">
+        <x:v>喜歡的卡通</x:v>
+      </x:c>
+      <x:c r="E36" s="11" t="str">
+        <x:v>電話號碼</x:v>
+      </x:c>
+      <x:c r="F36" s="11" t="str">
+        <x:v>最喜歡的水果</x:v>
+      </x:c>
+      <x:c r="G36" s="11" t="str"/>
+      <x:c r="H36" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I36" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J36" s="11" t="str"/>
+      <x:c r="K36" s="12" t="str">
+        <x:v>電話號碼可能讓陌生人聯絡到你，屬於應謹慎保護的個人資料。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="78" customHeight="1">
+      <x:c r="A37" s="10" t="str">
+        <x:v>陌生帳號詢問你的住址時，哪一個回應最安全？</x:v>
+      </x:c>
+      <x:c r="B37" s="11" t="str">
+        <x:v>Multiple Choice</x:v>
+      </x:c>
+      <x:c r="C37" s="11" t="str">
+        <x:v>先問對方住哪裡交換</x:v>
+      </x:c>
+      <x:c r="D37" s="11" t="str">
+        <x:v>只提供附近地標</x:v>
+      </x:c>
+      <x:c r="E37" s="11" t="str">
+        <x:v>請朋友代為回答</x:v>
+      </x:c>
+      <x:c r="F37" s="11" t="str">
+        <x:v>不提供，停止對話並告訴可信任的大人</x:v>
+      </x:c>
+      <x:c r="G37" s="11" t="str"/>
+      <x:c r="H37" s="11" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I37" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J37" s="11" t="str"/>
+      <x:c r="K37" s="12" t="str">
+        <x:v>不提供住址並求助可信任的大人，可以減少個資被濫用的風險。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="78" customHeight="1">
+      <x:c r="A38" s="10" t="str">
+        <x:v>留言送出前，可以用哪三個問題檢查？</x:v>
+      </x:c>
+      <x:c r="B38" s="11" t="str">
+        <x:v>Multiple Choice</x:v>
+      </x:c>
+      <x:c r="C38" s="11" t="str">
+        <x:v>夠快嗎？夠酸嗎？會紅嗎？</x:v>
+      </x:c>
+      <x:c r="D38" s="11" t="str">
+        <x:v>大家按讚嗎？有趣嗎？刺激嗎？</x:v>
+      </x:c>
+      <x:c r="E38" s="11" t="str">
+        <x:v>可以匿名嗎？可以刪掉嗎？可以轉傳嗎？</x:v>
+      </x:c>
+      <x:c r="F38" s="11" t="str">
+        <x:v>是真的嗎？必要嗎？尊重嗎？</x:v>
+      </x:c>
+      <x:c r="G38" s="11" t="str"/>
+      <x:c r="H38" s="11" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I38" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J38" s="11" t="str"/>
+      <x:c r="K38" s="12" t="str">
+        <x:v>留言前三問能幫助我們降低誤會與傷害：內容是否真實、是否必要、是否尊重。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="78" customHeight="1">
+      <x:c r="A39" s="10" t="str">
+        <x:v>留言前，若內容可能讓對方受傷，你可以怎麼做？</x:v>
+      </x:c>
+      <x:c r="B39" s="11" t="str">
+        <x:v>Multiple Choice</x:v>
+      </x:c>
+      <x:c r="C39" s="11" t="str">
+        <x:v>先停下來重寫，或選擇不送出</x:v>
+      </x:c>
+      <x:c r="D39" s="11" t="str">
+        <x:v>加上更多嘲笑</x:v>
+      </x:c>
+      <x:c r="E39" s="11" t="str">
+        <x:v>標註更多人圍觀</x:v>
+      </x:c>
+      <x:c r="F39" s="11" t="str">
+        <x:v>用匿名帳號送出</x:v>
+      </x:c>
+      <x:c r="G39" s="11" t="str"/>
+      <x:c r="H39" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I39" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J39" s="11" t="str"/>
+      <x:c r="K39" s="12" t="str">
+        <x:v>數位同理包含停下來評估影響，必要時重寫或不送出。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="78" customHeight="1">
+      <x:c r="A40" s="10" t="str">
+        <x:v>看到朋友發出可能受傷的留言時，怎麼回應較合適？</x:v>
+      </x:c>
+      <x:c r="B40" s="11" t="str">
+        <x:v>Multiple Choice</x:v>
+      </x:c>
+      <x:c r="C40" s="11" t="str">
+        <x:v>公開留言責備他</x:v>
+      </x:c>
+      <x:c r="D40" s="11" t="str">
+        <x:v>私下關心並視需要陪他找大人</x:v>
+      </x:c>
+      <x:c r="E40" s="11" t="str">
+        <x:v>截圖轉傳給全班</x:v>
+      </x:c>
+      <x:c r="F40" s="11" t="str">
+        <x:v>假裝沒看到</x:v>
+      </x:c>
+      <x:c r="G40" s="11" t="str"/>
+      <x:c r="H40" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I40" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J40" s="11" t="str"/>
+      <x:c r="K40" s="12" t="str">
+        <x:v>私下關心可以降低尷尬；若涉及安全疑慮，應陪同尋求可信任大人協助。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="78" customHeight="1">
+      <x:c r="A41" s="10" t="str">
+        <x:v>使用平板後，哪一個訊號提醒你需要休息？</x:v>
+      </x:c>
+      <x:c r="B41" s="11" t="str">
+        <x:v>Multiple Choice</x:v>
+      </x:c>
+      <x:c r="C41" s="11" t="str">
+        <x:v>眼睛疲累</x:v>
+      </x:c>
+      <x:c r="D41" s="11" t="str">
+        <x:v>以上都可能</x:v>
+      </x:c>
+      <x:c r="E41" s="11" t="str">
+        <x:v>睡不著</x:v>
+      </x:c>
+      <x:c r="F41" s="11" t="str">
+        <x:v>心情變差</x:v>
+      </x:c>
+      <x:c r="G41" s="11" t="str"/>
+      <x:c r="H41" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I41" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J41" s="11" t="str"/>
+      <x:c r="K41" s="12" t="str">
+        <x:v>身體和情緒訊號都值得注意；可以關閉通知、固定休息，並安排不使用螢幕的替代活動。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="78" customHeight="1">
+      <x:c r="A42" s="10" t="str">
+        <x:v>使用平板一段時間後，哪一個休息安排較實際？</x:v>
+      </x:c>
+      <x:c r="B42" s="11" t="str">
+        <x:v>Multiple Choice</x:v>
+      </x:c>
+      <x:c r="C42" s="11" t="str">
+        <x:v>一直滑到眼睛痛</x:v>
+      </x:c>
+      <x:c r="D42" s="11" t="str">
+        <x:v>關掉聲音但繼續看</x:v>
+      </x:c>
+      <x:c r="E42" s="11" t="str">
+        <x:v>離開螢幕、看看遠處並活動身體</x:v>
+      </x:c>
+      <x:c r="F42" s="11" t="str">
+        <x:v>熬夜補看所有內容</x:v>
+      </x:c>
+      <x:c r="G42" s="11" t="str"/>
+      <x:c r="H42" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I42" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J42" s="11" t="str"/>
+      <x:c r="K42" s="12" t="str">
+        <x:v>固定離開螢幕、看遠處和活動身體，有助於照顧身心狀態。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="78" customHeight="1">
+      <x:c r="A43" s="10" t="str">
+        <x:v>想建立數位平衡時，哪一個目標最可行？</x:v>
+      </x:c>
+      <x:c r="B43" s="11" t="str">
+        <x:v>Multiple Choice</x:v>
+      </x:c>
+      <x:c r="C43" s="11" t="str">
+        <x:v>永遠不再使用任何科技</x:v>
+      </x:c>
+      <x:c r="D43" s="11" t="str">
+        <x:v>每次都使用到凌晨</x:v>
+      </x:c>
+      <x:c r="E43" s="11" t="str">
+        <x:v>要求全家照自己的規則</x:v>
+      </x:c>
+      <x:c r="F43" s="11" t="str">
+        <x:v>每天晚餐時把通知關閉 20 分鐘</x:v>
+      </x:c>
+      <x:c r="G43" s="11" t="str"/>
+      <x:c r="H43" s="11" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I43" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J43" s="11" t="str"/>
+      <x:c r="K43" s="12" t="str">
+        <x:v>具體且能近期開始的小目標，比完全禁止或不切實際的要求更容易持續。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="78" customHeight="1">
+      <x:c r="A44" s="10" t="str">
+        <x:v>遇到可疑連結，第一步應該做什麼？</x:v>
+      </x:c>
+      <x:c r="B44" s="11" t="str">
+        <x:v>Multiple Choice</x:v>
+      </x:c>
+      <x:c r="C44" s="11" t="str">
+        <x:v>先停下來，不點開、不輸入資料</x:v>
+      </x:c>
+      <x:c r="D44" s="11" t="str">
+        <x:v>好奇地點開看看</x:v>
+      </x:c>
+      <x:c r="E44" s="11" t="str">
+        <x:v>轉傳給同學測試</x:v>
+      </x:c>
+      <x:c r="F44" s="11" t="str">
+        <x:v>輸入帳號密碼確認</x:v>
+      </x:c>
+      <x:c r="G44" s="11" t="str"/>
+      <x:c r="H44" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I44" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J44" s="11" t="str"/>
+      <x:c r="K44" s="12" t="str">
+        <x:v>可疑連結先不點、不輸入資料，保留訊息並找可信任的大人或正式管道確認。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="78" customHeight="1">
+      <x:c r="A45" s="10" t="str">
+        <x:v>遇到要求輸入密碼的陌生頁面，哪一個做法最安全？</x:v>
+      </x:c>
+      <x:c r="B45" s="11" t="str">
+        <x:v>Multiple Choice</x:v>
+      </x:c>
+      <x:c r="C45" s="11" t="str">
+        <x:v>先關閉頁面，不輸入資料並找大人確認</x:v>
+      </x:c>
+      <x:c r="D45" s="11" t="str">
+        <x:v>輸入常用密碼試試看</x:v>
+      </x:c>
+      <x:c r="E45" s="11" t="str">
+        <x:v>轉傳給同學點開</x:v>
+      </x:c>
+      <x:c r="F45" s="11" t="str">
+        <x:v>先填資料再檢查</x:v>
+      </x:c>
+      <x:c r="G45" s="11" t="str"/>
+      <x:c r="H45" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I45" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J45" s="11" t="str"/>
+      <x:c r="K45" s="12" t="str">
+        <x:v>陌生頁面不輸入帳密，先關閉並找可信任大人或正式管道確認。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="78" customHeight="1">
+      <x:c r="A46" s="10" t="str">
+        <x:v>收到可疑連結後，哪一項紀錄可能有助於求助？</x:v>
+      </x:c>
+      <x:c r="B46" s="11" t="str">
+        <x:v>Multiple Choice</x:v>
+      </x:c>
+      <x:c r="C46" s="11" t="str">
+        <x:v>把連結轉給更多人</x:v>
+      </x:c>
+      <x:c r="D46" s="11" t="str">
+        <x:v>保留訊息、網址或畫面截圖</x:v>
+      </x:c>
+      <x:c r="E46" s="11" t="str">
+        <x:v>只記住自己的猜測</x:v>
+      </x:c>
+      <x:c r="F46" s="11" t="str">
+        <x:v>刪除所有內容</x:v>
+      </x:c>
+      <x:c r="G46" s="11" t="str"/>
+      <x:c r="H46" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I46" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J46" s="11" t="str"/>
+      <x:c r="K46" s="12" t="str">
+        <x:v>保留必要紀錄能幫助可信任大人或平台了解情況並採取處理。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="78" customHeight="1">
+      <x:c r="A47" s="10" t="str">
+        <x:v>想到考試或升學時，哪一項可能是壓力訊號？</x:v>
+      </x:c>
+      <x:c r="B47" s="11" t="str">
+        <x:v>Multiple Choice</x:v>
+      </x:c>
+      <x:c r="C47" s="11" t="str">
+        <x:v>胃不舒服</x:v>
+      </x:c>
+      <x:c r="D47" s="11" t="str">
+        <x:v>睡不好</x:v>
+      </x:c>
+      <x:c r="E47" s="11" t="str">
+        <x:v>以上都可能</x:v>
+      </x:c>
+      <x:c r="F47" s="11" t="str">
+        <x:v>一直擔心來不及</x:v>
+      </x:c>
+      <x:c r="G47" s="11" t="str"/>
+      <x:c r="H47" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I47" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J47" s="11" t="str"/>
+      <x:c r="K47" s="12" t="str">
+        <x:v>壓力可能同時出現在身體、睡眠和想法；先辨認訊號，再把事情分成可控制與暫時不可控制。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="78" customHeight="1">
+      <x:c r="A48" s="10" t="str">
+        <x:v>壓力出現時，哪一種想法比較能幫助自己？</x:v>
+      </x:c>
+      <x:c r="B48" s="11" t="str">
+        <x:v>Multiple Choice</x:v>
+      </x:c>
+      <x:c r="C48" s="11" t="str">
+        <x:v>我一定要一次全部完成</x:v>
+      </x:c>
+      <x:c r="D48" s="11" t="str">
+        <x:v>只要緊張就是我很差</x:v>
+      </x:c>
+      <x:c r="E48" s="11" t="str">
+        <x:v>我可以先處理一件現在做得到的事</x:v>
+      </x:c>
+      <x:c r="F48" s="11" t="str">
+        <x:v>我不能向任何人求助</x:v>
+      </x:c>
+      <x:c r="G48" s="11" t="str"/>
+      <x:c r="H48" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I48" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J48" s="11" t="str"/>
+      <x:c r="K48" s="12" t="str">
+        <x:v>把壓力拆成現在做得到的一小步，能增加掌控感，也保留求助選項。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="78" customHeight="1">
+      <x:c r="A49" s="10" t="str">
+        <x:v>當壓力影響睡眠或日常很久時，可以怎麼做？</x:v>
+      </x:c>
+      <x:c r="B49" s="11" t="str">
+        <x:v>Multiple Choice</x:v>
+      </x:c>
+      <x:c r="C49" s="11" t="str">
+        <x:v>只責怪自己</x:v>
+      </x:c>
+      <x:c r="D49" s="11" t="str">
+        <x:v>完全不吃不睡</x:v>
+      </x:c>
+      <x:c r="E49" s="11" t="str">
+        <x:v>假裝什麼都沒發生</x:v>
+      </x:c>
+      <x:c r="F49" s="11" t="str">
+        <x:v>告訴可信任的大人，一起找適合的支持</x:v>
+      </x:c>
+      <x:c r="G49" s="11" t="str"/>
+      <x:c r="H49" s="11" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I49" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J49" s="11" t="str"/>
+      <x:c r="K49" s="12" t="str">
+        <x:v>持續影響生活的壓力值得被看見，找可信任大人一起尋求支持是負責任的做法。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="78" customHeight="1">
+      <x:c r="A50" s="10" t="str">
+        <x:v>「我要變厲害」可以改成哪一種比較可行的目標？</x:v>
+      </x:c>
+      <x:c r="B50" s="11" t="str">
+        <x:v>Multiple Choice</x:v>
+      </x:c>
+      <x:c r="C50" s="11" t="str">
+        <x:v>永遠第一名</x:v>
+      </x:c>
+      <x:c r="D50" s="11" t="str">
+        <x:v>不要失敗</x:v>
+      </x:c>
+      <x:c r="E50" s="11" t="str">
+        <x:v>讓所有人都滿意</x:v>
+      </x:c>
+      <x:c r="F50" s="11" t="str">
+        <x:v>今天完成 15 分鐘複習</x:v>
+      </x:c>
+      <x:c r="G50" s="11" t="str"/>
+      <x:c r="H50" s="11" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I50" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J50" s="11" t="str"/>
+      <x:c r="K50" s="12" t="str">
+        <x:v>可行目標要具體、能在近期開始；把大目標拆成今天的一小步，較容易看見進展。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="78" customHeight="1">
+      <x:c r="A51" s="10" t="str">
+        <x:v>把大目標拆小時，哪一項最像可執行的小步驟？</x:v>
+      </x:c>
+      <x:c r="B51" s="11" t="str">
+        <x:v>Multiple Choice</x:v>
+      </x:c>
+      <x:c r="C51" s="11" t="str">
+        <x:v>今晚先整理明天要讀的兩頁內容</x:v>
+      </x:c>
+      <x:c r="D51" s="11" t="str">
+        <x:v>我要立刻變成最厲害的人</x:v>
+      </x:c>
+      <x:c r="E51" s="11" t="str">
+        <x:v>我不能有任何錯誤</x:v>
+      </x:c>
+      <x:c r="F51" s="11" t="str">
+        <x:v>我要讓所有人滿意</x:v>
+      </x:c>
+      <x:c r="G51" s="11" t="str"/>
+      <x:c r="H51" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I51" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J51" s="11" t="str"/>
+      <x:c r="K51" s="12" t="str">
+        <x:v>具體、短期且可開始的小步驟，比模糊或不可能控制的目標更容易行動。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="78" customHeight="1">
+      <x:c r="A52" s="10" t="str">
+        <x:v>如果原定計畫被打斷，哪一種備案比較有幫助？</x:v>
+      </x:c>
+      <x:c r="B52" s="11" t="str">
+        <x:v>Multiple Choice</x:v>
+      </x:c>
+      <x:c r="C52" s="11" t="str">
+        <x:v>直接放棄所有計畫</x:v>
+      </x:c>
+      <x:c r="D52" s="11" t="str">
+        <x:v>改到明天固定的 15 分鐘完成</x:v>
+      </x:c>
+      <x:c r="E52" s="11" t="str">
+        <x:v>責怪打斷你的人</x:v>
+      </x:c>
+      <x:c r="F52" s="11" t="str">
+        <x:v>把時間加到完全不休息</x:v>
+      </x:c>
+      <x:c r="G52" s="11" t="str"/>
+      <x:c r="H52" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I52" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J52" s="11" t="str"/>
+      <x:c r="K52" s="12" t="str">
+        <x:v>備案讓行動可以調整，不必因一次中斷就把整個目標判定為失敗。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="78" customHeight="1">
+      <x:c r="A53" s="10" t="str">
+        <x:v>把「我就是不行」改成哪一句支持自己的話？</x:v>
+      </x:c>
+      <x:c r="B53" s="11" t="str">
+        <x:v>Multiple Choice</x:v>
+      </x:c>
+      <x:c r="C53" s="11" t="str">
+        <x:v>我現在還不會，但我可以先試一小步</x:v>
+      </x:c>
+      <x:c r="D53" s="11" t="str">
+        <x:v>我永遠不可能學會</x:v>
+      </x:c>
+      <x:c r="E53" s="11" t="str">
+        <x:v>別人都比我好</x:v>
+      </x:c>
+      <x:c r="F53" s="11" t="str">
+        <x:v>算了，完全不要做</x:v>
+      </x:c>
+      <x:c r="G53" s="11" t="str"/>
+      <x:c r="H53" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I53" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J53" s="11" t="str"/>
+      <x:c r="K53" s="12" t="str">
+        <x:v>成長語句不否認困難，而是把注意力放回目前能學習或嘗試的下一步。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="78" customHeight="1">
+      <x:c r="A54" s="10" t="str">
+        <x:v>哪一句話比較像支持自己的成長語句？</x:v>
+      </x:c>
+      <x:c r="B54" s="11" t="str">
+        <x:v>Multiple Choice</x:v>
+      </x:c>
+      <x:c r="C54" s="11" t="str">
+        <x:v>我永遠都做不到</x:v>
+      </x:c>
+      <x:c r="D54" s="11" t="str">
+        <x:v>別人一定比我好</x:v>
+      </x:c>
+      <x:c r="E54" s="11" t="str">
+        <x:v>我現在還不熟悉，但可以再練習一次</x:v>
+      </x:c>
+      <x:c r="F54" s="11" t="str">
+        <x:v>做不好就不要再試</x:v>
+      </x:c>
+      <x:c r="G54" s="11" t="str"/>
+      <x:c r="H54" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I54" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J54" s="11" t="str"/>
+      <x:c r="K54" s="12" t="str">
+        <x:v>成長語句承認目前困難，也把注意力放回可以嘗試的下一步。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="78" customHeight="1">
+      <x:c r="A55" s="10" t="str">
+        <x:v>自我支持時，哪一種說法最貼近事實？</x:v>
+      </x:c>
+      <x:c r="B55" s="11" t="str">
+        <x:v>Multiple Choice</x:v>
+      </x:c>
+      <x:c r="C55" s="11" t="str">
+        <x:v>我只要想開就會立刻成功</x:v>
+      </x:c>
+      <x:c r="D55" s="11" t="str">
+        <x:v>我不需要任何幫助</x:v>
+      </x:c>
+      <x:c r="E55" s="11" t="str">
+        <x:v>失敗表示我沒有能力</x:v>
+      </x:c>
+      <x:c r="F55" s="11" t="str">
+        <x:v>這次很難，但我可以找方法或請人陪我練習</x:v>
+      </x:c>
+      <x:c r="G55" s="11" t="str"/>
+      <x:c r="H55" s="11" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I55" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J55" s="11" t="str"/>
+      <x:c r="K55" s="12" t="str">
+        <x:v>支持自己不是保證立刻成功，而是承認困難並尋找方法、練習或協助。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="78" customHeight="1">
+      <x:c r="A56" s="10" t="str">
+        <x:v>遇到壓力時，什麼樣的大人可以成為支持者？</x:v>
+      </x:c>
+      <x:c r="B56" s="11" t="str">
+        <x:v>Multiple Choice</x:v>
+      </x:c>
+      <x:c r="C56" s="11" t="str">
+        <x:v>只要求你忍耐的人</x:v>
+      </x:c>
+      <x:c r="D56" s="11" t="str">
+        <x:v>願意聽、尊重界線並一起找方法的人</x:v>
+      </x:c>
+      <x:c r="E56" s="11" t="str">
+        <x:v>會把秘密公開的人</x:v>
+      </x:c>
+      <x:c r="F56" s="11" t="str">
+        <x:v>完全不聽你說的人</x:v>
+      </x:c>
+      <x:c r="G56" s="11" t="str"/>
+      <x:c r="H56" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I56" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J56" s="11" t="str"/>
+      <x:c r="K56" s="12" t="str">
+        <x:v>支持者不一定直接替你解決，但會願意聽、尊重界線，必要時陪你找合適的協助。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="78" customHeight="1">
+      <x:c r="A57" s="10" t="str">
+        <x:v>判斷一位支持者是否安全時，可以觀察什麼？</x:v>
+      </x:c>
+      <x:c r="B57" s="11" t="str">
+        <x:v>Multiple Choice</x:v>
+      </x:c>
+      <x:c r="C57" s="11" t="str">
+        <x:v>他願意聽、尊重界線，也會在需要時陪你找協助</x:v>
+      </x:c>
+      <x:c r="D57" s="11" t="str">
+        <x:v>他要求你永遠保守危險秘密</x:v>
+      </x:c>
+      <x:c r="E57" s="11" t="str">
+        <x:v>他常用威脅讓你照做</x:v>
+      </x:c>
+      <x:c r="F57" s="11" t="str">
+        <x:v>他把你的困擾公開取笑</x:v>
+      </x:c>
+      <x:c r="G57" s="11" t="str"/>
+      <x:c r="H57" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I57" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J57" s="11" t="str"/>
+      <x:c r="K57" s="12" t="str">
+        <x:v>安全支持者會聆聽、尊重界線，遇到安全問題也願意協助連結適當資源。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="78" customHeight="1">
+      <x:c r="A58" s="10" t="str">
+        <x:v>向支持者說明需要時，哪一句開頭比較有幫助？</x:v>
+      </x:c>
+      <x:c r="B58" s="11" t="str">
+        <x:v>Multiple Choice</x:v>
+      </x:c>
+      <x:c r="C58" s="11" t="str">
+        <x:v>你一定要立刻替我解決</x:v>
+      </x:c>
+      <x:c r="D58" s="11" t="str">
+        <x:v>我最近遇到一件困擾，想請你先聽我說</x:v>
+      </x:c>
+      <x:c r="E58" s="11" t="str">
+        <x:v>我什麼都不想說但你要懂</x:v>
+      </x:c>
+      <x:c r="F58" s="11" t="str">
+        <x:v>這都不重要不用聽</x:v>
+      </x:c>
+      <x:c r="G58" s="11" t="str"/>
+      <x:c r="H58" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I58" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J58" s="11" t="str"/>
+      <x:c r="K58" s="12" t="str">
+        <x:v>清楚說明自己需要先被聆聽，有助於支持者理解並一起找適合的下一步。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="78" customHeight="1">
+      <x:c r="A59" s="10" t="str">
+        <x:v>課程結束後，你想把哪一個方法帶回生活？</x:v>
+      </x:c>
+      <x:c r="B59" s="11" t="str">
+        <x:v>Multiple Choice</x:v>
+      </x:c>
+      <x:c r="C59" s="11" t="str">
+        <x:v>先辨認情緒和身體訊號</x:v>
+      </x:c>
+      <x:c r="D59" s="11" t="str">
+        <x:v>遇到困擾時找可信任的大人</x:v>
+      </x:c>
+      <x:c r="E59" s="11" t="str">
+        <x:v>以上都可以，選一個明天先試</x:v>
+      </x:c>
+      <x:c r="F59" s="11" t="str">
+        <x:v>先查證再轉傳訊息</x:v>
+      </x:c>
+      <x:c r="G59" s="11" t="str"/>
+      <x:c r="H59" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I59" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J59" s="11" t="str"/>
+      <x:c r="K59" s="12" t="str">
         <x:v>SEL 的重點不是一次做到完美，而是遇到變化時，知道可以重新辨認、選擇與求助。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="78" customHeight="1">
+      <x:c r="A60" s="10" t="str">
+        <x:v>回顧 20 節課時，哪一組能力可以互相連結？</x:v>
+      </x:c>
+      <x:c r="B60" s="11" t="str">
+        <x:v>Multiple Choice</x:v>
+      </x:c>
+      <x:c r="C60" s="11" t="str">
+        <x:v>只能選一種能力</x:v>
+      </x:c>
+      <x:c r="D60" s="11" t="str">
+        <x:v>只有考試時才有用</x:v>
+      </x:c>
+      <x:c r="E60" s="11" t="str">
+        <x:v>辨識、調節、求助與行動可以一起使用</x:v>
+      </x:c>
+      <x:c r="F60" s="11" t="str">
+        <x:v>遇到問題只能自己處理</x:v>
+      </x:c>
+      <x:c r="G60" s="11" t="str"/>
+      <x:c r="H60" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I60" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J60" s="11" t="str"/>
+      <x:c r="K60" s="12" t="str">
+        <x:v>SEL 能力可以依情境互相配合，先辨識，再調節、求助並採取下一步行動。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="78" customHeight="1">
+      <x:c r="A61" s="10" t="str">
+        <x:v>為下一站行動設定目標時，哪一項內容最完整？</x:v>
+      </x:c>
+      <x:c r="B61" s="11" t="str">
+        <x:v>Multiple Choice</x:v>
+      </x:c>
+      <x:c r="C61" s="11" t="str">
+        <x:v>只有一句很大的口號</x:v>
+      </x:c>
+      <x:c r="D61" s="11" t="str">
+        <x:v>只寫別人應該怎麼做</x:v>
+      </x:c>
+      <x:c r="E61" s="11" t="str">
+        <x:v>完全不需要時間或方法</x:v>
+      </x:c>
+      <x:c r="F61" s="11" t="str">
+        <x:v>一個小步驟、一個備案和一位支持者</x:v>
+      </x:c>
+      <x:c r="G61" s="11" t="str"/>
+      <x:c r="H61" s="11" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I61" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J61" s="11" t="str"/>
+      <x:c r="K61" s="12" t="str">
+        <x:v>行動卡包含小步驟、備案與支持者，能讓目標更具體也更有彈性。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb1d2b9f497304122"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc1d0004253234947"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1048,11 +2334,21 @@
       <x:c r="C2" s="11" t="str">
         <x:v>辨識當下情緒，不要求分享個人秘密。</x:v>
       </x:c>
-      <x:c r="D2" s="11" t="str"/>
-      <x:c r="E2" s="11" t="str"/>
-      <x:c r="F2" s="11" t="str"/>
-      <x:c r="G2" s="11" t="str"/>
-      <x:c r="H2" s="11" t="str"/>
+      <x:c r="D2" s="11" t="str">
+        <x:v>陰天</x:v>
+      </x:c>
+      <x:c r="E2" s="11" t="str">
+        <x:v>晴天</x:v>
+      </x:c>
+      <x:c r="F2" s="11" t="str">
+        <x:v>下雨</x:v>
+      </x:c>
+      <x:c r="G2" s="11" t="str">
+        <x:v>雷雨</x:v>
+      </x:c>
+      <x:c r="H2" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="I2" s="11" t="n">
         <x:v>30</x:v>
       </x:c>
@@ -1062,183 +2358,185 @@
     </x:row>
     <x:row r="3" ht="60" customHeight="1">
       <x:c r="A3" s="11" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="B3" s="11" t="str">
-        <x:v>身體訊號</x:v>
+        <x:v>情緒偵探</x:v>
       </x:c>
       <x:c r="C3" s="11" t="str">
-        <x:v>辨識情緒升溫時的身體線索。</x:v>
+        <x:v>把模糊的心情轉成可以觀察的線索。</x:v>
       </x:c>
       <x:c r="D3" s="11" t="str">
-        <x:v>心跳變快</x:v>
+        <x:v>我現在有點焦躁，肩膀也很緊</x:v>
       </x:c>
       <x:c r="E3" s="11" t="str">
-        <x:v>手心出汗</x:v>
+        <x:v>我沒事啦</x:v>
       </x:c>
       <x:c r="F3" s="11" t="str">
-        <x:v>肩膀變緊</x:v>
+        <x:v>大家都很煩</x:v>
       </x:c>
       <x:c r="G3" s="11" t="str">
-        <x:v>以上都可能</x:v>
+        <x:v>反正就是不好</x:v>
       </x:c>
       <x:c r="H3" s="11" t="n">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I3" s="11" t="n">
         <x:v>30</x:v>
       </x:c>
       <x:c r="J3" s="11" t="str">
-        <x:v>教師可追問：你會用哪一種安全方法讓自己穩下來？</x:v>
+        <x:v>把「不好」改成一句更具體的描述。</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="60" customHeight="1">
       <x:c r="A4" s="11" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="B4" s="11" t="str">
-        <x:v>生理期照顧</x:v>
+        <x:v>情緒偵探</x:v>
       </x:c>
       <x:c r="C4" s="11" t="str">
-        <x:v>練習青春期與生理期的尊重和求助。</x:v>
+        <x:v>練習在不確定時保留探索空間。</x:v>
       </x:c>
       <x:c r="D4" s="11" t="str">
-        <x:v>大聲詢問細節</x:v>
+        <x:v>立刻責怪自己</x:v>
       </x:c>
       <x:c r="E4" s="11" t="str">
-        <x:v>取笑對方</x:v>
+        <x:v>停一下，觀察身體和想法</x:v>
       </x:c>
       <x:c r="F4" s="11" t="str">
-        <x:v>安靜陪伴並通知可信任的大人</x:v>
+        <x:v>逼自己馬上說出答案</x:v>
       </x:c>
       <x:c r="G4" s="11" t="str">
-        <x:v>拍照傳到群組</x:v>
+        <x:v>假裝完全沒感覺</x:v>
       </x:c>
       <x:c r="H4" s="11" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="I4" s="11" t="n">
         <x:v>30</x:v>
       </x:c>
       <x:c r="J4" s="11" t="str">
-        <x:v>教師可追問：如果對方說想自己安靜一下，我們可以怎麼做？</x:v>
+        <x:v>可以用哪一個身體訊號開始觀察？</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="60" customHeight="1">
       <x:c r="A5" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B5" s="11" t="str">
+        <x:v>身體訊號</x:v>
+      </x:c>
+      <x:c r="C5" s="11" t="str">
+        <x:v>辨識情緒升溫時的身體線索。</x:v>
+      </x:c>
+      <x:c r="D5" s="11" t="str">
+        <x:v>心跳變快</x:v>
+      </x:c>
+      <x:c r="E5" s="11" t="str">
+        <x:v>手心出汗</x:v>
+      </x:c>
+      <x:c r="F5" s="11" t="str">
+        <x:v>肩膀變緊</x:v>
+      </x:c>
+      <x:c r="G5" s="11" t="str">
+        <x:v>以上都可能</x:v>
+      </x:c>
+      <x:c r="H5" s="11" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B5" s="11" t="str">
-        <x:v>情緒升溫</x:v>
-      </x:c>
-      <x:c r="C5" s="11" t="str">
-        <x:v>察覺需要暫停的時機。</x:v>
-      </x:c>
-      <x:c r="D5" s="11" t="str">
-        <x:v>沒有固定答案，察覺自己需要時就可以停</x:v>
-      </x:c>
-      <x:c r="E5" s="11" t="str">
-        <x:v>1 度</x:v>
-      </x:c>
-      <x:c r="F5" s="11" t="str">
-        <x:v>2 度</x:v>
-      </x:c>
-      <x:c r="G5" s="11" t="str">
-        <x:v>3 度以上</x:v>
-      </x:c>
-      <x:c r="H5" s="11" t="str"/>
       <x:c r="I5" s="11" t="n">
         <x:v>30</x:v>
       </x:c>
       <x:c r="J5" s="11" t="str">
-        <x:v>教師可追問：你的安全暫停方法有哪些？</x:v>
+        <x:v>教師可追問：你會用哪一種安全方法讓自己穩下來？</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="60" customHeight="1">
       <x:c r="A6" s="11" t="n">
-        <x:v>5</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="B6" s="11" t="str">
-        <x:v>求助入口</x:v>
+        <x:v>身體訊號</x:v>
       </x:c>
       <x:c r="C6" s="11" t="str">
-        <x:v>建立可信任的求助入口。</x:v>
+        <x:v>辨識緊張時可能出現的身體反應。</x:v>
       </x:c>
       <x:c r="D6" s="11" t="str">
-        <x:v>完全不告訴任何人</x:v>
+        <x:v>突然長出翅膀</x:v>
       </x:c>
       <x:c r="E6" s="11" t="str">
-        <x:v>只在網路上找陌生人</x:v>
+        <x:v>完全不需要休息</x:v>
       </x:c>
       <x:c r="F6" s="11" t="str">
-        <x:v>責怪自己不夠勇敢</x:v>
+        <x:v>呼吸變快或變淺</x:v>
       </x:c>
       <x:c r="G6" s="11" t="str">
-        <x:v>可信任的導師、家人、校護或輔導老師</x:v>
+        <x:v>一定會發燒</x:v>
       </x:c>
       <x:c r="H6" s="11" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="I6" s="11" t="n">
         <x:v>30</x:v>
       </x:c>
       <x:c r="J6" s="11" t="str">
-        <x:v>教師可追問：如果第一位大人沒空，你還能找誰？</x:v>
+        <x:v>你會選擇哪一種安全方法調節呼吸？</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="60" customHeight="1">
       <x:c r="A7" s="11" t="n">
-        <x:v>6</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="B7" s="11" t="str">
-        <x:v>朋友不同</x:v>
+        <x:v>身體訊號</x:v>
       </x:c>
       <x:c r="C7" s="11" t="str">
-        <x:v>尊重友誼中的差異。</x:v>
+        <x:v>把身體線索連結到安全調節行動。</x:v>
       </x:c>
       <x:c r="D7" s="11" t="str">
-        <x:v>逼對方改變</x:v>
+        <x:v>繼續硬撐到受不了</x:v>
       </x:c>
       <x:c r="E7" s="11" t="str">
-        <x:v>說出自己的喜好，也聽聽對方的想法</x:v>
+        <x:v>把責任推給別人</x:v>
       </x:c>
       <x:c r="F7" s="11" t="str">
-        <x:v>嘲笑對方</x:v>
+        <x:v>用傷害自己的方式發洩</x:v>
       </x:c>
       <x:c r="G7" s="11" t="str">
-        <x:v>假裝自己什麼都喜歡</x:v>
+        <x:v>先停下來，慢慢呼吸並觀察需要</x:v>
       </x:c>
       <x:c r="H7" s="11" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="I7" s="11" t="n">
         <x:v>30</x:v>
       </x:c>
       <x:c r="J7" s="11" t="str">
-        <x:v>教師可追問：如何約定輪流選擇？</x:v>
+        <x:v>為自己選一個可以在教室使用的暫停方法。</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="60" customHeight="1">
       <x:c r="A8" s="11" t="n">
-        <x:v>7</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="B8" s="11" t="str">
-        <x:v>界線訊號</x:v>
+        <x:v>生理期照顧</x:v>
       </x:c>
       <x:c r="C8" s="11" t="str">
-        <x:v>練習影像與個人界線。</x:v>
+        <x:v>練習青春期與生理期的尊重和求助。</x:v>
       </x:c>
       <x:c r="D8" s="11" t="str">
-        <x:v>好啦，大家都傳了</x:v>
+        <x:v>大聲詢問細節</x:v>
       </x:c>
       <x:c r="E8" s="11" t="str">
-        <x:v>你不傳我就取笑你</x:v>
+        <x:v>取笑對方</x:v>
       </x:c>
       <x:c r="F8" s="11" t="str">
-        <x:v>我不想分享這張照片，請不要傳</x:v>
+        <x:v>安靜陪伴並通知可信任的大人</x:v>
       </x:c>
       <x:c r="G8" s="11" t="str">
-        <x:v>先傳給陌生人問問看</x:v>
+        <x:v>拍照傳到群組</x:v>
       </x:c>
       <x:c r="H8" s="11" t="n">
         <x:v>3</x:v>
@@ -1247,30 +2545,30 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="J8" s="11" t="str">
-        <x:v>教師可追問：如果對方繼續要求，你的下一步是什麼？</x:v>
+        <x:v>教師可追問：如果對方說想自己安靜一下，我們可以怎麼做？</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="60" customHeight="1">
       <x:c r="A9" s="11" t="n">
-        <x:v>8</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="B9" s="11" t="str">
-        <x:v>衝突暫停</x:v>
+        <x:v>生理期照顧</x:v>
       </x:c>
       <x:c r="C9" s="11" t="str">
-        <x:v>練習衝突中的暫停與修復。</x:v>
+        <x:v>建立尊重身體差異的班級語言。</x:v>
       </x:c>
       <x:c r="D9" s="11" t="str">
-        <x:v>深呼吸並暫時離開刺激</x:v>
+        <x:v>尊重差異，不拿別人的身體開玩笑</x:v>
       </x:c>
       <x:c r="E9" s="11" t="str">
-        <x:v>繼續大喊</x:v>
+        <x:v>比較誰變化最快</x:v>
       </x:c>
       <x:c r="F9" s="11" t="str">
-        <x:v>推人</x:v>
+        <x:v>替別人公開說明</x:v>
       </x:c>
       <x:c r="G9" s="11" t="str">
-        <x:v>立刻把爭吵內容轉傳</x:v>
+        <x:v>用綽號取笑對方</x:v>
       </x:c>
       <x:c r="H9" s="11" t="n">
         <x:v>1</x:v>
@@ -1279,84 +2577,94 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="J9" s="11" t="str">
-        <x:v>教師可追問：回到對話時，可以先說哪一句話？</x:v>
+        <x:v>如果聽到取笑身體的話，可以怎麼回應？</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="60" customHeight="1">
       <x:c r="A10" s="11" t="n">
-        <x:v>9</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="B10" s="11" t="str">
-        <x:v>團體參與</x:v>
+        <x:v>生理期照顧</x:v>
       </x:c>
       <x:c r="C10" s="11" t="str">
-        <x:v>練習不強迫的團體邀請。</x:v>
-      </x:c>
-      <x:c r="D10" s="11" t="str"/>
-      <x:c r="E10" s="11" t="str"/>
-      <x:c r="F10" s="11" t="str"/>
-      <x:c r="G10" s="11" t="str"/>
-      <x:c r="H10" s="11" t="str"/>
+        <x:v>練習保護隱私的同理協助。</x:v>
+      </x:c>
+      <x:c r="D10" s="11" t="str">
+        <x:v>大聲問全班誰需要</x:v>
+      </x:c>
+      <x:c r="E10" s="11" t="str">
+        <x:v>低調提供資訊或陪同找可信任的大人</x:v>
+      </x:c>
+      <x:c r="F10" s="11" t="str">
+        <x:v>拍照記錄後分享</x:v>
+      </x:c>
+      <x:c r="G10" s="11" t="str">
+        <x:v>叫對方自己想辦法</x:v>
+      </x:c>
+      <x:c r="H10" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="I10" s="11" t="n">
         <x:v>30</x:v>
       </x:c>
       <x:c r="J10" s="11" t="str">
-        <x:v>教師可追問：小組還能怎麼分配角色，讓大家參與？</x:v>
+        <x:v>怎麼做可以讓對方感到被尊重？</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="60" customHeight="1">
       <x:c r="A11" s="11" t="n">
-        <x:v>10</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="B11" s="11" t="str">
-        <x:v>人際回應</x:v>
+        <x:v>情緒升溫</x:v>
       </x:c>
       <x:c r="C11" s="11" t="str">
-        <x:v>整合表達、拒絕與決定的方法。</x:v>
+        <x:v>察覺需要暫停的時機。</x:v>
       </x:c>
       <x:c r="D11" s="11" t="str">
-        <x:v>只要朋友開心就好</x:v>
+        <x:v>沒有固定答案，察覺自己需要時就可以停</x:v>
       </x:c>
       <x:c r="E11" s="11" t="str">
-        <x:v>別人怎麼做我就怎麼做</x:v>
+        <x:v>1 度</x:v>
       </x:c>
       <x:c r="F11" s="11" t="str">
-        <x:v>答應後再說</x:v>
+        <x:v>2 度</x:v>
       </x:c>
       <x:c r="G11" s="11" t="str">
-        <x:v>我的感受、我的界線和可能的結果</x:v>
+        <x:v>3 度以上</x:v>
       </x:c>
       <x:c r="H11" s="11" t="n">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I11" s="11" t="n">
         <x:v>30</x:v>
       </x:c>
       <x:c r="J11" s="11" t="str">
-        <x:v>教師可追問：你可以用哪一句話爭取思考時間？</x:v>
+        <x:v>教師可追問：你的安全暫停方法有哪些？</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="60" customHeight="1">
       <x:c r="A12" s="11" t="n">
-        <x:v>11</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="B12" s="11" t="str">
-        <x:v>資訊查證</x:v>
+        <x:v>情緒升溫</x:v>
       </x:c>
       <x:c r="C12" s="11" t="str">
-        <x:v>使用來源、日期、證據與目的查證訊息。</x:v>
+        <x:v>辨識需要暫停的心理與行為線索。</x:v>
       </x:c>
       <x:c r="D12" s="11" t="str">
-        <x:v>來源</x:v>
+        <x:v>覺得自己很平靜</x:v>
       </x:c>
       <x:c r="E12" s="11" t="str">
-        <x:v>日期</x:v>
+        <x:v>正在專心聽課</x:v>
       </x:c>
       <x:c r="F12" s="11" t="str">
-        <x:v>以上都要查</x:v>
+        <x:v>開始想大喊或做出衝動決定</x:v>
       </x:c>
       <x:c r="G12" s="11" t="str">
-        <x:v>證據</x:v>
+        <x:v>已經完成整理</x:v>
       </x:c>
       <x:c r="H12" s="11" t="n">
         <x:v>3</x:v>
@@ -1365,62 +2673,62 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="J12" s="11" t="str">
-        <x:v>教師可追問：哪一個官方或可信來源可以比對？</x:v>
+        <x:v>你可以用哪個手勢或暗號提醒自己？</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="60" customHeight="1">
       <x:c r="A13" s="11" t="n">
-        <x:v>12</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="B13" s="11" t="str">
-        <x:v>個資保護</x:v>
+        <x:v>情緒升溫</x:v>
       </x:c>
       <x:c r="C13" s="11" t="str">
-        <x:v>辨識個人資料與安全處理流程。</x:v>
+        <x:v>把暫停連結到後續選擇。</x:v>
       </x:c>
       <x:c r="D13" s="11" t="str">
-        <x:v>住址</x:v>
+        <x:v>立刻回去爭輸贏</x:v>
       </x:c>
       <x:c r="E13" s="11" t="str">
-        <x:v>喜歡的顏色</x:v>
+        <x:v>把對方的話公開</x:v>
       </x:c>
       <x:c r="F13" s="11" t="str">
-        <x:v>喜歡的遊戲角色</x:v>
+        <x:v>完全不必理會任何人</x:v>
       </x:c>
       <x:c r="G13" s="11" t="str">
-        <x:v>喜歡的食物</x:v>
+        <x:v>確認自己已比較穩定，再選擇說法或求助</x:v>
       </x:c>
       <x:c r="H13" s="11" t="n">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="I13" s="11" t="n">
         <x:v>30</x:v>
       </x:c>
       <x:c r="J13" s="11" t="str">
-        <x:v>教師可追問：除了不回覆，還能做哪三件事？</x:v>
+        <x:v>回到對話時可以先說哪一句？</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="60" customHeight="1">
       <x:c r="A14" s="11" t="n">
-        <x:v>13</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="B14" s="11" t="str">
-        <x:v>留言三秒</x:v>
+        <x:v>求助入口</x:v>
       </x:c>
       <x:c r="C14" s="11" t="str">
-        <x:v>練習數位同理與負責任留言。</x:v>
+        <x:v>建立可信任的求助入口。</x:v>
       </x:c>
       <x:c r="D14" s="11" t="str">
-        <x:v>夠快嗎？夠酸嗎？會紅嗎？</x:v>
+        <x:v>完全不告訴任何人</x:v>
       </x:c>
       <x:c r="E14" s="11" t="str">
-        <x:v>大家按讚嗎？有趣嗎？刺激嗎？</x:v>
+        <x:v>只在網路上找陌生人</x:v>
       </x:c>
       <x:c r="F14" s="11" t="str">
-        <x:v>可以匿名嗎？可以刪掉嗎？可以轉傳嗎？</x:v>
+        <x:v>責怪自己不夠勇敢</x:v>
       </x:c>
       <x:c r="G14" s="11" t="str">
-        <x:v>是真的嗎？必要嗎？尊重嗎？</x:v>
+        <x:v>可信任的導師、家人、校護或輔導老師</x:v>
       </x:c>
       <x:c r="H14" s="11" t="n">
         <x:v>4</x:v>
@@ -1429,213 +2737,1517 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="J14" s="11" t="str">
-        <x:v>教師可追問：把一句容易傷人的話改成尊重說法。</x:v>
+        <x:v>教師可追問：如果第一位大人沒空，你還能找誰？</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="60" customHeight="1">
       <x:c r="A15" s="11" t="n">
-        <x:v>14</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="B15" s="11" t="str">
-        <x:v>數位平衡</x:v>
+        <x:v>求助入口</x:v>
       </x:c>
       <x:c r="C15" s="11" t="str">
-        <x:v>觀察科技使用後的身心狀態。</x:v>
+        <x:v>練習讓求助訊息具體可理解。</x:v>
       </x:c>
       <x:c r="D15" s="11" t="str">
-        <x:v>眼睛疲累</x:v>
+        <x:v>說明發生什麼、何時發生，以及自己需要什麼</x:v>
       </x:c>
       <x:c r="E15" s="11" t="str">
-        <x:v>以上都可能</x:v>
+        <x:v>只說「你自己猜」</x:v>
       </x:c>
       <x:c r="F15" s="11" t="str">
-        <x:v>睡不著</x:v>
+        <x:v>先責怪自己</x:v>
       </x:c>
       <x:c r="G15" s="11" t="str">
-        <x:v>心情變差</x:v>
-      </x:c>
-      <x:c r="H15" s="11" t="str"/>
+        <x:v>完全不提供線索</x:v>
+      </x:c>
+      <x:c r="H15" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="I15" s="11" t="n">
         <x:v>30</x:v>
       </x:c>
       <x:c r="J15" s="11" t="str">
-        <x:v>教師可追問：你想為自己設定哪一個可行的休息提醒？</x:v>
+        <x:v>試著用一句話說出你需要的協助。</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="60" customHeight="1">
       <x:c r="A16" s="11" t="n">
-        <x:v>15</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="B16" s="11" t="str">
-        <x:v>網路闖關</x:v>
+        <x:v>求助入口</x:v>
       </x:c>
       <x:c r="C16" s="11" t="str">
-        <x:v>練習陌生連結的安全處理。</x:v>
+        <x:v>建立多一個求助選項的思考。</x:v>
       </x:c>
       <x:c r="D16" s="11" t="str">
-        <x:v>先停下來，不點開、不輸入資料</x:v>
+        <x:v>就此放棄</x:v>
       </x:c>
       <x:c r="E16" s="11" t="str">
-        <x:v>好奇地點開看看</x:v>
+        <x:v>再找另一位可信任的大人，持續求助</x:v>
       </x:c>
       <x:c r="F16" s="11" t="str">
-        <x:v>轉傳給同學測試</x:v>
+        <x:v>把事情傳給陌生人</x:v>
       </x:c>
       <x:c r="G16" s="11" t="str">
-        <x:v>輸入帳號密碼確認</x:v>
+        <x:v>責怪自己不值得幫忙</x:v>
       </x:c>
       <x:c r="H16" s="11" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="I16" s="11" t="n">
         <x:v>30</x:v>
       </x:c>
       <x:c r="J16" s="11" t="str">
-        <x:v>教師可追問：哪些線索會讓你覺得連結可疑？</x:v>
+        <x:v>你的第二位支持者可能是誰？</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="60" customHeight="1">
       <x:c r="A17" s="11" t="n">
-        <x:v>16</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="B17" s="11" t="str">
-        <x:v>壓力訊號</x:v>
+        <x:v>朋友不同</x:v>
       </x:c>
       <x:c r="C17" s="11" t="str">
-        <x:v>辨識升學與考試壓力的身心訊號。</x:v>
-      </x:c>
-      <x:c r="D17" s="11" t="str"/>
-      <x:c r="E17" s="11" t="str"/>
-      <x:c r="F17" s="11" t="str"/>
-      <x:c r="G17" s="11" t="str"/>
-      <x:c r="H17" s="11" t="str"/>
+        <x:v>尊重友誼中的差異。</x:v>
+      </x:c>
+      <x:c r="D17" s="11" t="str">
+        <x:v>逼對方改變</x:v>
+      </x:c>
+      <x:c r="E17" s="11" t="str">
+        <x:v>說出自己的喜好，也聽聽對方的想法</x:v>
+      </x:c>
+      <x:c r="F17" s="11" t="str">
+        <x:v>嘲笑對方</x:v>
+      </x:c>
+      <x:c r="G17" s="11" t="str">
+        <x:v>假裝自己什麼都喜歡</x:v>
+      </x:c>
+      <x:c r="H17" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="I17" s="11" t="n">
         <x:v>30</x:v>
       </x:c>
       <x:c r="J17" s="11" t="str">
-        <x:v>教師可追問：今天能做的一小步是什麼？</x:v>
+        <x:v>教師可追問：如何約定輪流選擇？</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="60" customHeight="1">
       <x:c r="A18" s="11" t="n">
-        <x:v>17</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="B18" s="11" t="str">
-        <x:v>下一小步</x:v>
+        <x:v>朋友不同</x:v>
       </x:c>
       <x:c r="C18" s="11" t="str">
-        <x:v>把焦慮轉成可執行的小目標。</x:v>
+        <x:v>練習尊重差異的對話。</x:v>
       </x:c>
       <x:c r="D18" s="11" t="str">
-        <x:v>永遠第一名</x:v>
+        <x:v>你怎麼這麼笨</x:v>
       </x:c>
       <x:c r="E18" s="11" t="str">
-        <x:v>不要失敗</x:v>
+        <x:v>你一定要照我的</x:v>
       </x:c>
       <x:c r="F18" s="11" t="str">
-        <x:v>讓所有人都滿意</x:v>
+        <x:v>我和你想法不同，但我們可以聽聽彼此</x:v>
       </x:c>
       <x:c r="G18" s="11" t="str">
-        <x:v>今天完成 15 分鐘複習</x:v>
+        <x:v>那就不要再當朋友</x:v>
       </x:c>
       <x:c r="H18" s="11" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="I18" s="11" t="n">
         <x:v>30</x:v>
       </x:c>
       <x:c r="J18" s="11" t="str">
-        <x:v>教師可追問：如果今天被打斷，你的備案是什麼？</x:v>
+        <x:v>把一句命令式說法改成邀請式說法。</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="60" customHeight="1">
       <x:c r="A19" s="11" t="n">
-        <x:v>18</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="B19" s="11" t="str">
-        <x:v>換個說法</x:v>
+        <x:v>朋友不同</x:v>
       </x:c>
       <x:c r="C19" s="11" t="str">
-        <x:v>練習成長語句與自我支持。</x:v>
-      </x:c>
-      <x:c r="D19" s="11" t="str"/>
-      <x:c r="E19" s="11" t="str"/>
-      <x:c r="F19" s="11" t="str"/>
-      <x:c r="G19" s="11" t="str"/>
-      <x:c r="H19" s="11" t="str"/>
+        <x:v>練習在差異中協商。</x:v>
+      </x:c>
+      <x:c r="D19" s="11" t="str">
+        <x:v>永遠只聽一個人的</x:v>
+      </x:c>
+      <x:c r="E19" s="11" t="str">
+        <x:v>誰大聲誰決定</x:v>
+      </x:c>
+      <x:c r="F19" s="11" t="str">
+        <x:v>完全不討論</x:v>
+      </x:c>
+      <x:c r="G19" s="11" t="str">
+        <x:v>輪流選擇，或一起找雙方都能接受的方案</x:v>
+      </x:c>
+      <x:c r="H19" s="11" t="n">
+        <x:v>4</x:v>
+      </x:c>
       <x:c r="I19" s="11" t="n">
         <x:v>30</x:v>
       </x:c>
       <x:c r="J19" s="11" t="str">
-        <x:v>教師可追問：你想把哪個「還不會」改成「先試試」？</x:v>
+        <x:v>小組可以訂什麼輪流規則？</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="60" customHeight="1">
       <x:c r="A20" s="11" t="n">
-        <x:v>19</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="B20" s="11" t="str">
-        <x:v>我的支持者</x:v>
+        <x:v>界線訊號</x:v>
       </x:c>
       <x:c r="C20" s="11" t="str">
-        <x:v>辨認安全且可信任的支持者。</x:v>
+        <x:v>練習影像與個人界線。</x:v>
       </x:c>
       <x:c r="D20" s="11" t="str">
-        <x:v>只要求你忍耐的人</x:v>
+        <x:v>好啦，大家都傳了</x:v>
       </x:c>
       <x:c r="E20" s="11" t="str">
-        <x:v>願意聽、尊重界線並一起找方法的人</x:v>
+        <x:v>你不傳我就取笑你</x:v>
       </x:c>
       <x:c r="F20" s="11" t="str">
-        <x:v>會把秘密公開的人</x:v>
+        <x:v>我不想分享這張照片，請不要傳</x:v>
       </x:c>
       <x:c r="G20" s="11" t="str">
-        <x:v>完全不聽你說的人</x:v>
+        <x:v>先傳給陌生人問問看</x:v>
       </x:c>
       <x:c r="H20" s="11" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="I20" s="11" t="n">
         <x:v>30</x:v>
       </x:c>
       <x:c r="J20" s="11" t="str">
-        <x:v>教師可追問：如果第一位大人不適合，你還能找誰？</x:v>
+        <x:v>教師可追問：如果對方繼續要求，你的下一步是什麼？</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="60" customHeight="1">
       <x:c r="A21" s="11" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B21" s="11" t="str">
+        <x:v>界線訊號</x:v>
+      </x:c>
+      <x:c r="C21" s="11" t="str">
+        <x:v>辨識影像分享中的界線與求助行動。</x:v>
+      </x:c>
+      <x:c r="D21" s="11" t="str">
+        <x:v>保留訊息、停止轉傳並找可信任的大人</x:v>
+      </x:c>
+      <x:c r="E21" s="11" t="str">
+        <x:v>照對方要求保守秘密</x:v>
+      </x:c>
+      <x:c r="F21" s="11" t="str">
+        <x:v>再轉給更多人</x:v>
+      </x:c>
+      <x:c r="G21" s="11" t="str">
+        <x:v>刪除所有證據後忍耐</x:v>
+      </x:c>
+      <x:c r="H21" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I21" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J21" s="11" t="str">
+        <x:v>除了截圖，你還可以找誰一起處理？</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="60" customHeight="1">
+      <x:c r="A22" s="11" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B22" s="11" t="str">
+        <x:v>界線訊號</x:v>
+      </x:c>
+      <x:c r="C22" s="11" t="str">
+        <x:v>練習清楚表達拒絕與求助。</x:v>
+      </x:c>
+      <x:c r="D22" s="11" t="str">
+        <x:v>你應該知道我不想要</x:v>
+      </x:c>
+      <x:c r="E22" s="11" t="str">
+        <x:v>我不願意，請停止；需要時我會找大人</x:v>
+      </x:c>
+      <x:c r="F22" s="11" t="str">
+        <x:v>隨便你啦</x:v>
+      </x:c>
+      <x:c r="G22" s="11" t="str">
+        <x:v>我先答應再後悔</x:v>
+      </x:c>
+      <x:c r="H22" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I22" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J22" s="11" t="str">
+        <x:v>用平靜聲音練習一次拒絕句。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="60" customHeight="1">
+      <x:c r="A23" s="11" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B23" s="11" t="str">
+        <x:v>衝突暫停</x:v>
+      </x:c>
+      <x:c r="C23" s="11" t="str">
+        <x:v>練習衝突中的暫停與修復。</x:v>
+      </x:c>
+      <x:c r="D23" s="11" t="str">
+        <x:v>深呼吸並暫時離開刺激</x:v>
+      </x:c>
+      <x:c r="E23" s="11" t="str">
+        <x:v>繼續大喊</x:v>
+      </x:c>
+      <x:c r="F23" s="11" t="str">
+        <x:v>推人</x:v>
+      </x:c>
+      <x:c r="G23" s="11" t="str">
+        <x:v>立刻把爭吵內容轉傳</x:v>
+      </x:c>
+      <x:c r="H23" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I23" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J23" s="11" t="str">
+        <x:v>教師可追問：回到對話時，可以先說哪一句話？</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="60" customHeight="1">
+      <x:c r="A24" s="11" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B24" s="11" t="str">
+        <x:v>衝突暫停</x:v>
+      </x:c>
+      <x:c r="C24" s="11" t="str">
+        <x:v>把衝突處理和安全判斷連結。</x:v>
+      </x:c>
+      <x:c r="D24" s="11" t="str">
+        <x:v>靠近對方繼續挑釁</x:v>
+      </x:c>
+      <x:c r="E24" s="11" t="str">
+        <x:v>立刻錄影上傳</x:v>
+      </x:c>
+      <x:c r="F24" s="11" t="str">
+        <x:v>先確認自己與他人都沒有受傷，再決定是否對話</x:v>
+      </x:c>
+      <x:c r="G24" s="11" t="str">
+        <x:v>用力推開對方</x:v>
+      </x:c>
+      <x:c r="H24" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I24" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J24" s="11" t="str">
+        <x:v>什麼情況下要直接找大人介入？</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="60" customHeight="1">
+      <x:c r="A25" s="11" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B25" s="11" t="str">
+        <x:v>衝突暫停</x:v>
+      </x:c>
+      <x:c r="C25" s="11" t="str">
+        <x:v>練習衝突後的修復語句。</x:v>
+      </x:c>
+      <x:c r="D25" s="11" t="str">
+        <x:v>都是你害的</x:v>
+      </x:c>
+      <x:c r="E25" s="11" t="str">
+        <x:v>你不准再提</x:v>
+      </x:c>
+      <x:c r="F25" s="11" t="str">
+        <x:v>我道歉但你不能有意見</x:v>
+      </x:c>
+      <x:c r="G25" s="11" t="str">
+        <x:v>我剛才的做法讓你不舒服，我想聽聽你的感受</x:v>
+      </x:c>
+      <x:c r="H25" s="11" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I25" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J25" s="11" t="str">
+        <x:v>這句話中哪一部分表示你願意聆聽？</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="60" customHeight="1">
+      <x:c r="A26" s="11" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B26" s="11" t="str">
+        <x:v>團體參與</x:v>
+      </x:c>
+      <x:c r="C26" s="11" t="str">
+        <x:v>練習不強迫的團體邀請。</x:v>
+      </x:c>
+      <x:c r="D26" s="11" t="str">
+        <x:v>你一定要現在回答</x:v>
+      </x:c>
+      <x:c r="E26" s="11" t="str">
+        <x:v>你想先聽聽他的想法嗎？也可以等一下再說</x:v>
+      </x:c>
+      <x:c r="F26" s="11" t="str">
+        <x:v>大家不要理他</x:v>
+      </x:c>
+      <x:c r="G26" s="11" t="str">
+        <x:v>替他直接決定</x:v>
+      </x:c>
+      <x:c r="H26" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I26" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J26" s="11" t="str">
+        <x:v>教師可追問：小組還能怎麼分配角色，讓大家參與？</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="60" customHeight="1">
+      <x:c r="A27" s="11" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B27" s="11" t="str">
+        <x:v>團體參與</x:v>
+      </x:c>
+      <x:c r="C27" s="11" t="str">
+        <x:v>設計保留選擇的參與邀請。</x:v>
+      </x:c>
+      <x:c r="D27" s="11" t="str">
+        <x:v>你想現在說，還是先用寫的？</x:v>
+      </x:c>
+      <x:c r="E27" s="11" t="str">
+        <x:v>你一定要說</x:v>
+      </x:c>
+      <x:c r="F27" s="11" t="str">
+        <x:v>不說就扣分</x:v>
+      </x:c>
+      <x:c r="G27" s="11" t="str">
+        <x:v>我替你回答</x:v>
+      </x:c>
+      <x:c r="H27" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I27" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J27" s="11" t="str">
+        <x:v>小組還能提供哪些參與方式？</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="60" customHeight="1">
+      <x:c r="A28" s="11" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B28" s="11" t="str">
+        <x:v>團體參與</x:v>
+      </x:c>
+      <x:c r="C28" s="11" t="str">
+        <x:v>練習以選擇支持團體參與。</x:v>
+      </x:c>
+      <x:c r="D28" s="11" t="str">
+        <x:v>直接替他決定全部工作</x:v>
+      </x:c>
+      <x:c r="E28" s="11" t="str">
+        <x:v>先詢問意願，再安排適合的角色</x:v>
+      </x:c>
+      <x:c r="F28" s="11" t="str">
+        <x:v>要求他代表全組發言</x:v>
+      </x:c>
+      <x:c r="G28" s="11" t="str">
+        <x:v>完全忽略他的想法</x:v>
+      </x:c>
+      <x:c r="H28" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I28" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J28" s="11" t="str">
+        <x:v>哪些角色不一定要公開發言？</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="60" customHeight="1">
+      <x:c r="A29" s="11" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B29" s="11" t="str">
+        <x:v>人際回應</x:v>
+      </x:c>
+      <x:c r="C29" s="11" t="str">
+        <x:v>整合表達、拒絕與決定的方法。</x:v>
+      </x:c>
+      <x:c r="D29" s="11" t="str">
+        <x:v>只要朋友開心就好</x:v>
+      </x:c>
+      <x:c r="E29" s="11" t="str">
+        <x:v>別人怎麼做我就怎麼做</x:v>
+      </x:c>
+      <x:c r="F29" s="11" t="str">
+        <x:v>答應後再說</x:v>
+      </x:c>
+      <x:c r="G29" s="11" t="str">
+        <x:v>我的感受、我的界線和可能的結果</x:v>
+      </x:c>
+      <x:c r="H29" s="11" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I29" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J29" s="11" t="str">
+        <x:v>教師可追問：你可以用哪一句話爭取思考時間？</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="60" customHeight="1">
+      <x:c r="A30" s="11" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B30" s="11" t="str">
+        <x:v>人際回應</x:v>
+      </x:c>
+      <x:c r="C30" s="11" t="str">
+        <x:v>整合界線表達與替代方案。</x:v>
+      </x:c>
+      <x:c r="D30" s="11" t="str">
+        <x:v>先答應再想辦法</x:v>
+      </x:c>
+      <x:c r="E30" s="11" t="str">
+        <x:v>先嘲笑對方</x:v>
+      </x:c>
+      <x:c r="F30" s="11" t="str">
+        <x:v>先說感受或界線，再說可以接受的替代方案</x:v>
+      </x:c>
+      <x:c r="G30" s="11" t="str">
+        <x:v>完全不回應</x:v>
+      </x:c>
+      <x:c r="H30" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I30" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J30" s="11" t="str">
+        <x:v>你能提出一個不傷害自己的替代方案嗎？</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="60" customHeight="1">
+      <x:c r="A31" s="11" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B31" s="11" t="str">
+        <x:v>人際回應</x:v>
+      </x:c>
+      <x:c r="C31" s="11" t="str">
+        <x:v>練習以感受和界線支持決定。</x:v>
+      </x:c>
+      <x:c r="D31" s="11" t="str">
+        <x:v>大家會不會都稱讚我？</x:v>
+      </x:c>
+      <x:c r="E31" s="11" t="str">
+        <x:v>最快可以結束嗎？</x:v>
+      </x:c>
+      <x:c r="F31" s="11" t="str">
+        <x:v>別人是否都這樣做？</x:v>
+      </x:c>
+      <x:c r="G31" s="11" t="str">
+        <x:v>這符合我的感受與界線嗎？</x:v>
+      </x:c>
+      <x:c r="H31" s="11" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I31" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J31" s="11" t="str">
+        <x:v>還可以問哪一個關於可能結果的問題？</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="60" customHeight="1">
+      <x:c r="A32" s="11" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B32" s="11" t="str">
+        <x:v>資訊查證</x:v>
+      </x:c>
+      <x:c r="C32" s="11" t="str">
+        <x:v>使用來源、日期、證據與目的查證訊息。</x:v>
+      </x:c>
+      <x:c r="D32" s="11" t="str">
+        <x:v>來源</x:v>
+      </x:c>
+      <x:c r="E32" s="11" t="str">
+        <x:v>日期</x:v>
+      </x:c>
+      <x:c r="F32" s="11" t="str">
+        <x:v>以上都要查</x:v>
+      </x:c>
+      <x:c r="G32" s="11" t="str">
+        <x:v>證據</x:v>
+      </x:c>
+      <x:c r="H32" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I32" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J32" s="11" t="str">
+        <x:v>教師可追問：哪一個官方或可信來源可以比對？</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="60" customHeight="1">
+      <x:c r="A33" s="11" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B33" s="11" t="str">
+        <x:v>資訊查證</x:v>
+      </x:c>
+      <x:c r="C33" s="11" t="str">
+        <x:v>辨識查證時的關鍵線索。</x:v>
+      </x:c>
+      <x:c r="D33" s="11" t="str">
+        <x:v>發布者是否可信、內容是否有日期與證據</x:v>
+      </x:c>
+      <x:c r="E33" s="11" t="str">
+        <x:v>標題是否夠生氣</x:v>
+      </x:c>
+      <x:c r="F33" s="11" t="str">
+        <x:v>轉發人數是否很多</x:v>
+      </x:c>
+      <x:c r="G33" s="11" t="str">
+        <x:v>圖片是否夠吸睛</x:v>
+      </x:c>
+      <x:c r="H33" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I33" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J33" s="11" t="str">
+        <x:v>你會用哪個正式來源交叉比對？</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="60" customHeight="1">
+      <x:c r="A34" s="11" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B34" s="11" t="str">
+        <x:v>資訊查證</x:v>
+      </x:c>
+      <x:c r="C34" s="11" t="str">
+        <x:v>練習查證前的暫停。</x:v>
+      </x:c>
+      <x:c r="D34" s="11" t="str">
+        <x:v>先轉傳再說</x:v>
+      </x:c>
+      <x:c r="E34" s="11" t="str">
+        <x:v>先暫停轉傳，查到可信資料再決定</x:v>
+      </x:c>
+      <x:c r="F34" s="11" t="str">
+        <x:v>只看留言猜測</x:v>
+      </x:c>
+      <x:c r="G34" s="11" t="str">
+        <x:v>把疑問改成肯定語氣</x:v>
+      </x:c>
+      <x:c r="H34" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I34" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J34" s="11" t="str">
+        <x:v>可以把「我聽說」改成哪種較誠實的說法？</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="60" customHeight="1">
+      <x:c r="A35" s="11" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B35" s="11" t="str">
+        <x:v>個資保護</x:v>
+      </x:c>
+      <x:c r="C35" s="11" t="str">
+        <x:v>辨識個人資料與安全處理流程。</x:v>
+      </x:c>
+      <x:c r="D35" s="11" t="str">
+        <x:v>住址</x:v>
+      </x:c>
+      <x:c r="E35" s="11" t="str">
+        <x:v>喜歡的顏色</x:v>
+      </x:c>
+      <x:c r="F35" s="11" t="str">
+        <x:v>喜歡的遊戲角色</x:v>
+      </x:c>
+      <x:c r="G35" s="11" t="str">
+        <x:v>喜歡的食物</x:v>
+      </x:c>
+      <x:c r="H35" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I35" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J35" s="11" t="str">
+        <x:v>教師可追問：除了不回覆，還能做哪三件事？</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="60" customHeight="1">
+      <x:c r="A36" s="11" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B36" s="11" t="str">
+        <x:v>個資保護</x:v>
+      </x:c>
+      <x:c r="C36" s="11" t="str">
+        <x:v>辨識需要保護的個人資料。</x:v>
+      </x:c>
+      <x:c r="D36" s="11" t="str">
+        <x:v>喜歡的顏色</x:v>
+      </x:c>
+      <x:c r="E36" s="11" t="str">
+        <x:v>喜歡的卡通</x:v>
+      </x:c>
+      <x:c r="F36" s="11" t="str">
+        <x:v>電話號碼</x:v>
+      </x:c>
+      <x:c r="G36" s="11" t="str">
+        <x:v>最喜歡的水果</x:v>
+      </x:c>
+      <x:c r="H36" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I36" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J36" s="11" t="str">
+        <x:v>還有哪些資料不適合公開在陌生網站？</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="60" customHeight="1">
+      <x:c r="A37" s="11" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B37" s="11" t="str">
+        <x:v>個資保護</x:v>
+      </x:c>
+      <x:c r="C37" s="11" t="str">
+        <x:v>練習面對個資索取的安全回應。</x:v>
+      </x:c>
+      <x:c r="D37" s="11" t="str">
+        <x:v>先問對方住哪裡交換</x:v>
+      </x:c>
+      <x:c r="E37" s="11" t="str">
+        <x:v>只提供附近地標</x:v>
+      </x:c>
+      <x:c r="F37" s="11" t="str">
+        <x:v>請朋友代為回答</x:v>
+      </x:c>
+      <x:c r="G37" s="11" t="str">
+        <x:v>不提供，停止對話並告訴可信任的大人</x:v>
+      </x:c>
+      <x:c r="H37" s="11" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I37" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J37" s="11" t="str">
+        <x:v>如果對方持續詢問，可以使用哪些平台功能？</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="60" customHeight="1">
+      <x:c r="A38" s="11" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B38" s="11" t="str">
+        <x:v>留言三秒</x:v>
+      </x:c>
+      <x:c r="C38" s="11" t="str">
+        <x:v>練習數位同理與負責任留言。</x:v>
+      </x:c>
+      <x:c r="D38" s="11" t="str">
+        <x:v>夠快嗎？夠酸嗎？會紅嗎？</x:v>
+      </x:c>
+      <x:c r="E38" s="11" t="str">
+        <x:v>大家按讚嗎？有趣嗎？刺激嗎？</x:v>
+      </x:c>
+      <x:c r="F38" s="11" t="str">
+        <x:v>可以匿名嗎？可以刪掉嗎？可以轉傳嗎？</x:v>
+      </x:c>
+      <x:c r="G38" s="11" t="str">
+        <x:v>是真的嗎？必要嗎？尊重嗎？</x:v>
+      </x:c>
+      <x:c r="H38" s="11" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I38" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J38" s="11" t="str">
+        <x:v>教師可追問：把一句容易傷人的話改成尊重說法。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="60" customHeight="1">
+      <x:c r="A39" s="11" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B39" s="11" t="str">
+        <x:v>留言三秒</x:v>
+      </x:c>
+      <x:c r="C39" s="11" t="str">
+        <x:v>練習留言前的同理判斷。</x:v>
+      </x:c>
+      <x:c r="D39" s="11" t="str">
+        <x:v>先停下來重寫，或選擇不送出</x:v>
+      </x:c>
+      <x:c r="E39" s="11" t="str">
+        <x:v>加上更多嘲笑</x:v>
+      </x:c>
+      <x:c r="F39" s="11" t="str">
+        <x:v>標註更多人圍觀</x:v>
+      </x:c>
+      <x:c r="G39" s="11" t="str">
+        <x:v>用匿名帳號送出</x:v>
+      </x:c>
+      <x:c r="H39" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I39" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J39" s="11" t="str">
+        <x:v>把傷人的詞換成描述事情的句子。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="60" customHeight="1">
+      <x:c r="A40" s="11" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B40" s="11" t="str">
+        <x:v>留言三秒</x:v>
+      </x:c>
+      <x:c r="C40" s="11" t="str">
+        <x:v>把數位同理連結到支持與求助。</x:v>
+      </x:c>
+      <x:c r="D40" s="11" t="str">
+        <x:v>公開留言責備他</x:v>
+      </x:c>
+      <x:c r="E40" s="11" t="str">
+        <x:v>私下關心並視需要陪他找大人</x:v>
+      </x:c>
+      <x:c r="F40" s="11" t="str">
+        <x:v>截圖轉傳給全班</x:v>
+      </x:c>
+      <x:c r="G40" s="11" t="str">
+        <x:v>假裝沒看到</x:v>
+      </x:c>
+      <x:c r="H40" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I40" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J40" s="11" t="str">
+        <x:v>什麼情況下需要立即找大人？</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="60" customHeight="1">
+      <x:c r="A41" s="11" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B41" s="11" t="str">
+        <x:v>數位平衡</x:v>
+      </x:c>
+      <x:c r="C41" s="11" t="str">
+        <x:v>觀察科技使用後的身心狀態。</x:v>
+      </x:c>
+      <x:c r="D41" s="11" t="str">
+        <x:v>眼睛疲累</x:v>
+      </x:c>
+      <x:c r="E41" s="11" t="str">
+        <x:v>以上都可能</x:v>
+      </x:c>
+      <x:c r="F41" s="11" t="str">
+        <x:v>睡不著</x:v>
+      </x:c>
+      <x:c r="G41" s="11" t="str">
+        <x:v>心情變差</x:v>
+      </x:c>
+      <x:c r="H41" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I41" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J41" s="11" t="str">
+        <x:v>教師可追問：你想為自己設定哪一個可行的休息提醒？</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="60" customHeight="1">
+      <x:c r="A42" s="11" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B42" s="11" t="str">
+        <x:v>數位平衡</x:v>
+      </x:c>
+      <x:c r="C42" s="11" t="str">
+        <x:v>把身體訊號轉成可行休息行動。</x:v>
+      </x:c>
+      <x:c r="D42" s="11" t="str">
+        <x:v>一直滑到眼睛痛</x:v>
+      </x:c>
+      <x:c r="E42" s="11" t="str">
+        <x:v>關掉聲音但繼續看</x:v>
+      </x:c>
+      <x:c r="F42" s="11" t="str">
+        <x:v>離開螢幕、看看遠處並活動身體</x:v>
+      </x:c>
+      <x:c r="G42" s="11" t="str">
+        <x:v>熬夜補看所有內容</x:v>
+      </x:c>
+      <x:c r="H42" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I42" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J42" s="11" t="str">
+        <x:v>你想設定什麼提醒幫助自己休息？</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="60" customHeight="1">
+      <x:c r="A43" s="11" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B43" s="11" t="str">
+        <x:v>數位平衡</x:v>
+      </x:c>
+      <x:c r="C43" s="11" t="str">
+        <x:v>練習設定具體可行的數位休息目標。</x:v>
+      </x:c>
+      <x:c r="D43" s="11" t="str">
+        <x:v>永遠不再使用任何科技</x:v>
+      </x:c>
+      <x:c r="E43" s="11" t="str">
+        <x:v>每次都使用到凌晨</x:v>
+      </x:c>
+      <x:c r="F43" s="11" t="str">
+        <x:v>要求全家照自己的規則</x:v>
+      </x:c>
+      <x:c r="G43" s="11" t="str">
+        <x:v>每天晚餐時把通知關閉 20 分鐘</x:v>
+      </x:c>
+      <x:c r="H43" s="11" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I43" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J43" s="11" t="str">
+        <x:v>你的目標何時開始、如何提醒？</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="60" customHeight="1">
+      <x:c r="A44" s="11" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B44" s="11" t="str">
+        <x:v>網路闖關</x:v>
+      </x:c>
+      <x:c r="C44" s="11" t="str">
+        <x:v>練習陌生連結的安全處理。</x:v>
+      </x:c>
+      <x:c r="D44" s="11" t="str">
+        <x:v>先停下來，不點開、不輸入資料</x:v>
+      </x:c>
+      <x:c r="E44" s="11" t="str">
+        <x:v>好奇地點開看看</x:v>
+      </x:c>
+      <x:c r="F44" s="11" t="str">
+        <x:v>轉傳給同學測試</x:v>
+      </x:c>
+      <x:c r="G44" s="11" t="str">
+        <x:v>輸入帳號密碼確認</x:v>
+      </x:c>
+      <x:c r="H44" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I44" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J44" s="11" t="str">
+        <x:v>教師可追問：哪些線索會讓你覺得連結可疑？</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="60" customHeight="1">
+      <x:c r="A45" s="11" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B45" s="11" t="str">
+        <x:v>網路闖關</x:v>
+      </x:c>
+      <x:c r="C45" s="11" t="str">
+        <x:v>練習處理索取帳密的可疑頁面。</x:v>
+      </x:c>
+      <x:c r="D45" s="11" t="str">
+        <x:v>先關閉頁面，不輸入資料並找大人確認</x:v>
+      </x:c>
+      <x:c r="E45" s="11" t="str">
+        <x:v>輸入常用密碼試試看</x:v>
+      </x:c>
+      <x:c r="F45" s="11" t="str">
+        <x:v>轉傳給同學點開</x:v>
+      </x:c>
+      <x:c r="G45" s="11" t="str">
+        <x:v>先填資料再檢查</x:v>
+      </x:c>
+      <x:c r="H45" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I45" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J45" s="11" t="str">
+        <x:v>哪些網址或訊息線索會讓你提高警覺？</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="60" customHeight="1">
+      <x:c r="A46" s="11" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B46" s="11" t="str">
+        <x:v>網路闖關</x:v>
+      </x:c>
+      <x:c r="C46" s="11" t="str">
+        <x:v>建立安全求助所需的紀錄習慣。</x:v>
+      </x:c>
+      <x:c r="D46" s="11" t="str">
+        <x:v>把連結轉給更多人</x:v>
+      </x:c>
+      <x:c r="E46" s="11" t="str">
+        <x:v>保留訊息、網址或畫面截圖</x:v>
+      </x:c>
+      <x:c r="F46" s="11" t="str">
+        <x:v>只記住自己的猜測</x:v>
+      </x:c>
+      <x:c r="G46" s="11" t="str">
+        <x:v>刪除所有內容</x:v>
+      </x:c>
+      <x:c r="H46" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I46" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J46" s="11" t="str">
+        <x:v>保留紀錄後，下一步可以找誰？</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="60" customHeight="1">
+      <x:c r="A47" s="11" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B47" s="11" t="str">
+        <x:v>壓力訊號</x:v>
+      </x:c>
+      <x:c r="C47" s="11" t="str">
+        <x:v>辨識升學與考試壓力的身心訊號。</x:v>
+      </x:c>
+      <x:c r="D47" s="11" t="str">
+        <x:v>胃不舒服</x:v>
+      </x:c>
+      <x:c r="E47" s="11" t="str">
+        <x:v>睡不好</x:v>
+      </x:c>
+      <x:c r="F47" s="11" t="str">
+        <x:v>以上都可能</x:v>
+      </x:c>
+      <x:c r="G47" s="11" t="str">
+        <x:v>一直擔心來不及</x:v>
+      </x:c>
+      <x:c r="H47" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I47" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J47" s="11" t="str">
+        <x:v>教師可追問：今天能做的一小步是什麼？</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="60" customHeight="1">
+      <x:c r="A48" s="11" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B48" s="11" t="str">
+        <x:v>壓力訊號</x:v>
+      </x:c>
+      <x:c r="C48" s="11" t="str">
+        <x:v>練習把壓力轉成可處理的小步驟。</x:v>
+      </x:c>
+      <x:c r="D48" s="11" t="str">
+        <x:v>我一定要一次全部完成</x:v>
+      </x:c>
+      <x:c r="E48" s="11" t="str">
+        <x:v>只要緊張就是我很差</x:v>
+      </x:c>
+      <x:c r="F48" s="11" t="str">
+        <x:v>我可以先處理一件現在做得到的事</x:v>
+      </x:c>
+      <x:c r="G48" s="11" t="str">
+        <x:v>我不能向任何人求助</x:v>
+      </x:c>
+      <x:c r="H48" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I48" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J48" s="11" t="str">
+        <x:v>今天最小、最可行的一步是什麼？</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="60" customHeight="1">
+      <x:c r="A49" s="11" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B49" s="11" t="str">
+        <x:v>壓力訊號</x:v>
+      </x:c>
+      <x:c r="C49" s="11" t="str">
+        <x:v>辨識需要進一步求助的壓力狀況。</x:v>
+      </x:c>
+      <x:c r="D49" s="11" t="str">
+        <x:v>只責怪自己</x:v>
+      </x:c>
+      <x:c r="E49" s="11" t="str">
+        <x:v>完全不吃不睡</x:v>
+      </x:c>
+      <x:c r="F49" s="11" t="str">
+        <x:v>假裝什麼都沒發生</x:v>
+      </x:c>
+      <x:c r="G49" s="11" t="str">
+        <x:v>告訴可信任的大人，一起找適合的支持</x:v>
+      </x:c>
+      <x:c r="H49" s="11" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I49" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J49" s="11" t="str">
+        <x:v>你願意先和哪一位大人說說看？</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="60" customHeight="1">
+      <x:c r="A50" s="11" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B50" s="11" t="str">
+        <x:v>下一小步</x:v>
+      </x:c>
+      <x:c r="C50" s="11" t="str">
+        <x:v>把焦慮轉成可執行的小目標。</x:v>
+      </x:c>
+      <x:c r="D50" s="11" t="str">
+        <x:v>永遠第一名</x:v>
+      </x:c>
+      <x:c r="E50" s="11" t="str">
+        <x:v>不要失敗</x:v>
+      </x:c>
+      <x:c r="F50" s="11" t="str">
+        <x:v>讓所有人都滿意</x:v>
+      </x:c>
+      <x:c r="G50" s="11" t="str">
+        <x:v>今天完成 15 分鐘複習</x:v>
+      </x:c>
+      <x:c r="H50" s="11" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I50" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J50" s="11" t="str">
+        <x:v>教師可追問：如果今天被打斷，你的備案是什麼？</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="60" customHeight="1">
+      <x:c r="A51" s="11" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B51" s="11" t="str">
+        <x:v>下一小步</x:v>
+      </x:c>
+      <x:c r="C51" s="11" t="str">
+        <x:v>練習把目標轉成近期行動。</x:v>
+      </x:c>
+      <x:c r="D51" s="11" t="str">
+        <x:v>今晚先整理明天要讀的兩頁內容</x:v>
+      </x:c>
+      <x:c r="E51" s="11" t="str">
+        <x:v>我要立刻變成最厲害的人</x:v>
+      </x:c>
+      <x:c r="F51" s="11" t="str">
+        <x:v>我不能有任何錯誤</x:v>
+      </x:c>
+      <x:c r="G51" s="11" t="str">
+        <x:v>我要讓所有人滿意</x:v>
+      </x:c>
+      <x:c r="H51" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I51" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J51" s="11" t="str">
+        <x:v>完成小步驟後，你要如何記錄進度？</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="60" customHeight="1">
+      <x:c r="A52" s="11" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B52" s="11" t="str">
+        <x:v>下一小步</x:v>
+      </x:c>
+      <x:c r="C52" s="11" t="str">
+        <x:v>建立可調整的行動備案。</x:v>
+      </x:c>
+      <x:c r="D52" s="11" t="str">
+        <x:v>直接放棄所有計畫</x:v>
+      </x:c>
+      <x:c r="E52" s="11" t="str">
+        <x:v>改到明天固定的 15 分鐘完成</x:v>
+      </x:c>
+      <x:c r="F52" s="11" t="str">
+        <x:v>責怪打斷你的人</x:v>
+      </x:c>
+      <x:c r="G52" s="11" t="str">
+        <x:v>把時間加到完全不休息</x:v>
+      </x:c>
+      <x:c r="H52" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I52" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J52" s="11" t="str">
+        <x:v>你的備案需要哪些提醒或支持？</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="60" customHeight="1">
+      <x:c r="A53" s="11" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B53" s="11" t="str">
+        <x:v>換個說法</x:v>
+      </x:c>
+      <x:c r="C53" s="11" t="str">
+        <x:v>練習成長語句與自我支持。</x:v>
+      </x:c>
+      <x:c r="D53" s="11" t="str">
+        <x:v>我現在還不會，但我可以先試一小步</x:v>
+      </x:c>
+      <x:c r="E53" s="11" t="str">
+        <x:v>我永遠不可能學會</x:v>
+      </x:c>
+      <x:c r="F53" s="11" t="str">
+        <x:v>別人都比我好</x:v>
+      </x:c>
+      <x:c r="G53" s="11" t="str">
+        <x:v>算了，完全不要做</x:v>
+      </x:c>
+      <x:c r="H53" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I53" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J53" s="11" t="str">
+        <x:v>教師可追問：你想把哪個「還不會」改成「先試試」？</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="60" customHeight="1">
+      <x:c r="A54" s="11" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B54" s="11" t="str">
+        <x:v>換個說法</x:v>
+      </x:c>
+      <x:c r="C54" s="11" t="str">
+        <x:v>練習用成長語句取代全盤否定。</x:v>
+      </x:c>
+      <x:c r="D54" s="11" t="str">
+        <x:v>我永遠都做不到</x:v>
+      </x:c>
+      <x:c r="E54" s="11" t="str">
+        <x:v>別人一定比我好</x:v>
+      </x:c>
+      <x:c r="F54" s="11" t="str">
+        <x:v>我現在還不熟悉，但可以再練習一次</x:v>
+      </x:c>
+      <x:c r="G54" s="11" t="str">
+        <x:v>做不好就不要再試</x:v>
+      </x:c>
+      <x:c r="H54" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I54" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J54" s="11" t="str">
+        <x:v>把一句「我不會」改成「我還在學」。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="60" customHeight="1">
+      <x:c r="A55" s="11" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B55" s="11" t="str">
+        <x:v>換個說法</x:v>
+      </x:c>
+      <x:c r="C55" s="11" t="str">
+        <x:v>建立務實而有支持性的自我對話。</x:v>
+      </x:c>
+      <x:c r="D55" s="11" t="str">
+        <x:v>我只要想開就會立刻成功</x:v>
+      </x:c>
+      <x:c r="E55" s="11" t="str">
+        <x:v>我不需要任何幫助</x:v>
+      </x:c>
+      <x:c r="F55" s="11" t="str">
+        <x:v>失敗表示我沒有能力</x:v>
+      </x:c>
+      <x:c r="G55" s="11" t="str">
+        <x:v>這次很難，但我可以找方法或請人陪我練習</x:v>
+      </x:c>
+      <x:c r="H55" s="11" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I55" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J55" s="11" t="str">
+        <x:v>你可以找誰陪你練習？</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="60" customHeight="1">
+      <x:c r="A56" s="11" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B56" s="11" t="str">
+        <x:v>我的支持者</x:v>
+      </x:c>
+      <x:c r="C56" s="11" t="str">
+        <x:v>辨認安全且可信任的支持者。</x:v>
+      </x:c>
+      <x:c r="D56" s="11" t="str">
+        <x:v>只要求你忍耐的人</x:v>
+      </x:c>
+      <x:c r="E56" s="11" t="str">
+        <x:v>願意聽、尊重界線並一起找方法的人</x:v>
+      </x:c>
+      <x:c r="F56" s="11" t="str">
+        <x:v>會把秘密公開的人</x:v>
+      </x:c>
+      <x:c r="G56" s="11" t="str">
+        <x:v>完全不聽你說的人</x:v>
+      </x:c>
+      <x:c r="H56" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I56" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J56" s="11" t="str">
+        <x:v>教師可追問：如果第一位大人不適合，你還能找誰？</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="60" customHeight="1">
+      <x:c r="A57" s="11" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B57" s="11" t="str">
+        <x:v>我的支持者</x:v>
+      </x:c>
+      <x:c r="C57" s="11" t="str">
+        <x:v>辨認安全支持者的特徵。</x:v>
+      </x:c>
+      <x:c r="D57" s="11" t="str">
+        <x:v>他願意聽、尊重界線，也會在需要時陪你找協助</x:v>
+      </x:c>
+      <x:c r="E57" s="11" t="str">
+        <x:v>他要求你永遠保守危險秘密</x:v>
+      </x:c>
+      <x:c r="F57" s="11" t="str">
+        <x:v>他常用威脅讓你照做</x:v>
+      </x:c>
+      <x:c r="G57" s="11" t="str">
+        <x:v>他把你的困擾公開取笑</x:v>
+      </x:c>
+      <x:c r="H57" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I57" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J57" s="11" t="str">
+        <x:v>如果不確定，可以和哪位大人一起判斷？</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="60" customHeight="1">
+      <x:c r="A58" s="11" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B58" s="11" t="str">
+        <x:v>我的支持者</x:v>
+      </x:c>
+      <x:c r="C58" s="11" t="str">
+        <x:v>練習向支持者開啟對話。</x:v>
+      </x:c>
+      <x:c r="D58" s="11" t="str">
+        <x:v>你一定要立刻替我解決</x:v>
+      </x:c>
+      <x:c r="E58" s="11" t="str">
+        <x:v>我最近遇到一件困擾，想請你先聽我說</x:v>
+      </x:c>
+      <x:c r="F58" s="11" t="str">
+        <x:v>我什麼都不想說但你要懂</x:v>
+      </x:c>
+      <x:c r="G58" s="11" t="str">
+        <x:v>這都不重要不用聽</x:v>
+      </x:c>
+      <x:c r="H58" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I58" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J58" s="11" t="str">
+        <x:v>你希望對方先聽、陪伴，還是一起想方法？</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="60" customHeight="1">
+      <x:c r="A59" s="11" t="n">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="B21" s="11" t="str">
+      <x:c r="B59" s="11" t="str">
         <x:v>下一站行動</x:v>
       </x:c>
-      <x:c r="C21" s="11" t="str">
+      <x:c r="C59" s="11" t="str">
         <x:v>把課堂策略轉成明天可開始的行動。</x:v>
       </x:c>
-      <x:c r="D21" s="11" t="str">
+      <x:c r="D59" s="11" t="str">
         <x:v>先辨認情緒和身體訊號</x:v>
       </x:c>
-      <x:c r="E21" s="11" t="str">
+      <x:c r="E59" s="11" t="str">
         <x:v>遇到困擾時找可信任的大人</x:v>
       </x:c>
-      <x:c r="F21" s="11" t="str">
+      <x:c r="F59" s="11" t="str">
         <x:v>以上都可以，選一個明天先試</x:v>
       </x:c>
-      <x:c r="G21" s="11" t="str">
+      <x:c r="G59" s="11" t="str">
         <x:v>先查證再轉傳訊息</x:v>
       </x:c>
-      <x:c r="H21" s="11" t="str"/>
-      <x:c r="I21" s="11" t="n">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="J21" s="11" t="str">
+      <x:c r="H59" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I59" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J59" s="11" t="str">
         <x:v>教師可追問：你明天準備在什麼時間第一次使用？</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="60" customHeight="1">
+      <x:c r="A60" s="11" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B60" s="11" t="str">
+        <x:v>下一站行動</x:v>
+      </x:c>
+      <x:c r="C60" s="11" t="str">
+        <x:v>整合課程中的 SEL 策略。</x:v>
+      </x:c>
+      <x:c r="D60" s="11" t="str">
+        <x:v>只能選一種能力</x:v>
+      </x:c>
+      <x:c r="E60" s="11" t="str">
+        <x:v>只有考試時才有用</x:v>
+      </x:c>
+      <x:c r="F60" s="11" t="str">
+        <x:v>辨識、調節、求助與行動可以一起使用</x:v>
+      </x:c>
+      <x:c r="G60" s="11" t="str">
+        <x:v>遇到問題只能自己處理</x:v>
+      </x:c>
+      <x:c r="H60" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I60" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J60" s="11" t="str">
+        <x:v>請舉一個你會先辨識再求助的情境。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="60" customHeight="1">
+      <x:c r="A61" s="11" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B61" s="11" t="str">
+        <x:v>下一站行動</x:v>
+      </x:c>
+      <x:c r="C61" s="11" t="str">
+        <x:v>完成可帶回生活的行動規劃。</x:v>
+      </x:c>
+      <x:c r="D61" s="11" t="str">
+        <x:v>只有一句很大的口號</x:v>
+      </x:c>
+      <x:c r="E61" s="11" t="str">
+        <x:v>只寫別人應該怎麼做</x:v>
+      </x:c>
+      <x:c r="F61" s="11" t="str">
+        <x:v>完全不需要時間或方法</x:v>
+      </x:c>
+      <x:c r="G61" s="11" t="str">
+        <x:v>一個小步驟、一個備案和一位支持者</x:v>
+      </x:c>
+      <x:c r="H61" s="11" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I61" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J61" s="11" t="str">
+        <x:v>你的行動卡第一步何時開始？</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0cded633fa694126"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfa6223b0b5374aff"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1667,7 +4279,7 @@
         <x:v>題型</x:v>
       </x:c>
       <x:c r="B3" s="7" t="str">
-        <x:v>20 題 Multiple Choice，每題 4 個選項，預設 30 秒。</x:v>
+        <x:v>60 題 Multiple Choice，每節課 3 題、每題 4 個選項與正確答案，預設 30 秒。</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="42" customHeight="1">

</xml_diff>